<commit_message>
napis losowania i etykieta linku Find out more, dopisane 4 zweryfikowane linki
</commit_message>
<xml_diff>
--- a/filmy.xlsx
+++ b/filmy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/96626423858cd10c/Studia ^M kursy/Github/Movie app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_2843028F942566422BD8D34292326807E4B775BE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DDB89CFE-7CD0-4C98-9521-64FAE784DECC}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_2843028F5F75A24349D9D357BABC0748EE37753E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{899B14A5-1DB6-4174-819F-9991B4F07F8F}"/>
   <bookViews>
     <workbookView xWindow="-51600" yWindow="0" windowWidth="25800" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="486">
   <si>
     <t>Tytuł</t>
   </si>
@@ -58,7 +58,7 @@
     <t>Leon Trystan</t>
   </si>
   <si>
-    <t>Śmiech</t>
+    <t>Komedia</t>
   </si>
   <si>
     <t>Adolf Dymsza w przebraniu, które ma rozstrzygnąć spór o spokój w kamienicy.</t>
@@ -67,6 +67,9 @@
     <t>Przedwojenna komedia o wojnie sąsiedzkiej prowadzonej przez sufit.</t>
   </si>
   <si>
+    <t>https://www.filmweb.pl/film/Pi%C4%99tro+wy%C5%BCej-1937-33181</t>
+  </si>
+  <si>
     <t>Znachor</t>
   </si>
   <si>
@@ -97,6 +100,9 @@
     <t>Przedwojenny musical o nauczycielu gimnastyki, pensji dla dziewcząt i piosence nie do wyrzucenia z głowy.</t>
   </si>
   <si>
+    <t>https://www.filmweb.pl/film/Zapomniana+melodia-1938-33183</t>
+  </si>
+  <si>
     <t>Włóczęgi</t>
   </si>
   <si>
@@ -145,7 +151,7 @@
     <t>Przygoda na Mariensztacie</t>
   </si>
   <si>
-    <t>Śmiech, PRL</t>
+    <t>Komedia, PRL</t>
   </si>
   <si>
     <t>Socrealizm w technikolorze, dziś oglądany jak eksponat.</t>
@@ -190,6 +196,9 @@
     <t>Powstańcy schodzą do kanałów i film zamienia się w powolne zejście bez wyjścia.</t>
   </si>
   <si>
+    <t>https://www.filmweb.pl/film/Kana%C5%82-1956-1117</t>
+  </si>
+  <si>
     <t>Pętla</t>
   </si>
   <si>
@@ -244,7 +253,7 @@
     <t>Eroica</t>
   </si>
   <si>
-    <t>Wojna, Śmiech</t>
+    <t>Wojna, Komedia</t>
   </si>
   <si>
     <t>Oficer ukryty w obozie, z którego wszyscy zrobili legendę.</t>
@@ -541,7 +550,7 @@
     <t>Jak rozpętałem drugą wojnę światową</t>
   </si>
   <si>
-    <t>Śmiech, Wojna</t>
+    <t>Komedia, Wojna</t>
   </si>
   <si>
     <t>Grzegorz Brzęczyszczykiewicz</t>
@@ -679,7 +688,7 @@
     <t>Wniebowzięci</t>
   </si>
   <si>
-    <t>Śmiech, Kino osobne</t>
+    <t>Komedia, Kino osobne</t>
   </si>
   <si>
     <t>Piwo pite na szczycie miasta, z którego wszystko wygląda inaczej.</t>
@@ -916,7 +925,7 @@
     <t>Juliusz Machulski</t>
   </si>
   <si>
-    <t>Kryminał, Śmiech</t>
+    <t>Kryminał, Komedia</t>
   </si>
   <si>
     <t>Kwinto z trąbką i plan skoku rozpisany co do sekundy.</t>
@@ -934,6 +943,9 @@
     <t>Trzy wersje jednego życia zależne od tego, czy bohater zdąży na pociąg.</t>
   </si>
   <si>
+    <t>https://www.filmweb.pl/film/Przypadek-1981-897</t>
+  </si>
+  <si>
     <t>Człowiek z żelaza</t>
   </si>
   <si>
@@ -961,7 +973,7 @@
     <t>Witold Leszczyński</t>
   </si>
   <si>
-    <t>Śmiech, Obyczajowe</t>
+    <t>Komedia, Obyczajowe</t>
   </si>
   <si>
     <t>Chłop, który boi się kosiarki bardziej niż diabła.</t>
@@ -1117,7 +1129,7 @@
     <t>Piłkarski poker</t>
   </si>
   <si>
-    <t>Śmiech, Kryminał</t>
+    <t>Komedia, Kryminał</t>
   </si>
   <si>
     <t>Narada w hotelowym pokoju, gdzie ustala się wynik przed pierwszym gwizdkiem.</t>
@@ -1291,7 +1303,7 @@
     <t>Marek Koterski</t>
   </si>
   <si>
-    <t>Śmiech, Egzystencjalne</t>
+    <t>Komedia, Egzystencjalne</t>
   </si>
   <si>
     <t>Poranna litania przy stole: kanapka, radio i lista pretensji do świata.</t>
@@ -1369,7 +1381,7 @@
     <t>Borys Lankosz</t>
   </si>
   <si>
-    <t>Śmiech, Kryminał, PRL</t>
+    <t>Komedia, Kryminał, PRL</t>
   </si>
   <si>
     <t>Czarno-biała Warszawa filmowana jak elegancka komedia kryminalna.</t>
@@ -1895,14 +1907,16 @@
       <c r="H2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="I2" s="1"/>
+      <c r="I2" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="3" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" s="1">
         <v>1937</v>
@@ -1911,25 +1925,25 @@
         <v>100</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" s="1">
         <v>1938</v>
@@ -1942,19 +1956,21 @@
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" s="1"/>
+        <v>24</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="5" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5" s="1">
         <v>1939</v>
@@ -1967,19 +1983,19 @@
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="I5" s="1"/>
     </row>
     <row r="6" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C6" s="1">
         <v>1946</v>
@@ -1988,23 +2004,23 @@
         <v>97</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I6" s="1"/>
     </row>
     <row r="7" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C7" s="1">
         <v>1948</v>
@@ -2013,23 +2029,23 @@
         <v>110</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="I7" s="1"/>
     </row>
     <row r="8" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C8" s="1">
         <v>1949</v>
@@ -2042,19 +2058,19 @@
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="I8" s="1"/>
     </row>
     <row r="9" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C9" s="1">
         <v>1954</v>
@@ -2063,23 +2079,23 @@
         <v>90</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I9" s="1"/>
     </row>
     <row r="10" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C10" s="1">
         <v>1955</v>
@@ -2088,23 +2104,23 @@
         <v>85</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F10" s="1"/>
       <c r="G10" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I10" s="1"/>
     </row>
     <row r="11" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C11" s="1">
         <v>1956</v>
@@ -2113,23 +2129,23 @@
         <v>95</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="I11" s="1"/>
     </row>
     <row r="12" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C12" s="1">
         <v>1957</v>
@@ -2138,23 +2154,25 @@
         <v>91</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="I12" s="1"/>
+        <v>56</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="13" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C13" s="1">
         <v>1957</v>
@@ -2163,23 +2181,23 @@
         <v>96</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="I13" s="1"/>
     </row>
     <row r="14" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C14" s="1">
         <v>1957</v>
@@ -2188,23 +2206,23 @@
         <v>82</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I14" s="1"/>
     </row>
     <row r="15" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C15" s="1">
         <v>1957</v>
@@ -2217,19 +2235,19 @@
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="I15" s="1"/>
     </row>
     <row r="16" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C16" s="1">
         <v>1958</v>
@@ -2238,23 +2256,23 @@
         <v>103</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="I16" s="1"/>
     </row>
     <row r="17" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C17" s="1">
         <v>1958</v>
@@ -2263,23 +2281,23 @@
         <v>83</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I17" s="1"/>
     </row>
     <row r="18" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C18" s="1">
         <v>1958</v>
@@ -2288,23 +2306,23 @@
         <v>66</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="I18" s="1"/>
     </row>
     <row r="19" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C19" s="1">
         <v>1958</v>
@@ -2313,23 +2331,23 @@
         <v>95</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="I19" s="1"/>
     </row>
     <row r="20" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C20" s="1">
         <v>1959</v>
@@ -2338,23 +2356,23 @@
         <v>93</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="I20" s="1"/>
     </row>
     <row r="21" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C21" s="1">
         <v>1959</v>
@@ -2363,23 +2381,23 @@
         <v>88</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="I21" s="1"/>
     </row>
     <row r="22" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C22" s="1">
         <v>1960</v>
@@ -2388,23 +2406,23 @@
         <v>166</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F22" s="1"/>
       <c r="G22" s="1" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="I22" s="1"/>
     </row>
     <row r="23" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C23" s="1">
         <v>1960</v>
@@ -2417,19 +2435,19 @@
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="I23" s="1"/>
     </row>
     <row r="24" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C24" s="1">
         <v>1960</v>
@@ -2438,23 +2456,23 @@
         <v>87</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F24" s="1"/>
       <c r="G24" s="1" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="I24" s="1"/>
     </row>
     <row r="25" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C25" s="1">
         <v>1960</v>
@@ -2463,23 +2481,23 @@
         <v>82</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F25" s="1"/>
       <c r="G25" s="1" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="I25" s="1"/>
     </row>
     <row r="26" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C26" s="1">
         <v>1961</v>
@@ -2488,23 +2506,23 @@
         <v>110</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F26" s="1"/>
       <c r="G26" s="1" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I26" s="1"/>
     </row>
     <row r="27" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C27" s="1">
         <v>1962</v>
@@ -2513,23 +2531,23 @@
         <v>94</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F27" s="1"/>
       <c r="G27" s="1" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="I27" s="1"/>
     </row>
     <row r="28" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C28" s="1">
         <v>1963</v>
@@ -2538,23 +2556,23 @@
         <v>97</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="F28" s="1"/>
       <c r="G28" s="1" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="I28" s="1"/>
     </row>
     <row r="29" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C29" s="1">
         <v>1963</v>
@@ -2563,23 +2581,23 @@
         <v>62</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F29" s="1"/>
       <c r="G29" s="1" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="I29" s="1"/>
     </row>
     <row r="30" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C30" s="1">
         <v>1964</v>
@@ -2588,23 +2606,23 @@
         <v>91</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="F30" s="1"/>
       <c r="G30" s="1" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="I30" s="1"/>
     </row>
     <row r="31" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C31" s="1">
         <v>1964</v>
@@ -2613,23 +2631,23 @@
         <v>76</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F31" s="1"/>
       <c r="G31" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="I31" s="1"/>
     </row>
     <row r="32" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C32" s="1">
         <v>1965</v>
@@ -2638,23 +2656,23 @@
         <v>182</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="F32" s="1"/>
       <c r="G32" s="1" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="I32" s="1"/>
     </row>
     <row r="33" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C33" s="1">
         <v>1965</v>
@@ -2663,23 +2681,23 @@
         <v>100</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="F33" s="1"/>
       <c r="G33" s="1" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="I33" s="1"/>
     </row>
     <row r="34" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C34" s="1">
         <v>1965</v>
@@ -2688,23 +2706,23 @@
         <v>77</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F34" s="1"/>
       <c r="G34" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I34" s="1"/>
     </row>
     <row r="35" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C35" s="1">
         <v>1965</v>
@@ -2713,23 +2731,23 @@
         <v>233</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="F35" s="1"/>
       <c r="G35" s="1" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="I35" s="1"/>
     </row>
     <row r="36" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C36" s="1">
         <v>1966</v>
@@ -2738,23 +2756,23 @@
         <v>175</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F36" s="1"/>
       <c r="G36" s="1" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C37" s="1">
         <v>1966</v>
@@ -2763,23 +2781,23 @@
         <v>83</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="F37" s="1"/>
       <c r="G37" s="1" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="I37" s="1"/>
     </row>
     <row r="38" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C38" s="1">
         <v>1967</v>
@@ -2791,20 +2809,20 @@
         <v>11</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="G38" s="1"/>
       <c r="H38" s="1" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="I38" s="1"/>
     </row>
     <row r="39" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="C39" s="1">
         <v>1967</v>
@@ -2813,23 +2831,23 @@
         <v>87</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F39" s="1"/>
       <c r="G39" s="1" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="I39" s="1"/>
     </row>
     <row r="40" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C40" s="1">
         <v>1968</v>
@@ -2838,23 +2856,23 @@
         <v>100</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F40" s="1"/>
       <c r="G40" s="1" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="I40" s="1"/>
     </row>
     <row r="41" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C41" s="1">
         <v>1968</v>
@@ -2863,23 +2881,23 @@
         <v>158</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F41" s="1"/>
       <c r="G41" s="1" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="I41" s="1"/>
     </row>
     <row r="42" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C42" s="1">
         <v>1969</v>
@@ -2888,23 +2906,23 @@
         <v>74</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F42" s="1"/>
       <c r="G42" s="1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="I42" s="1"/>
     </row>
     <row r="43" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C43" s="1">
         <v>1969</v>
@@ -2913,23 +2931,23 @@
         <v>100</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F43" s="1"/>
       <c r="G43" s="1" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="I43" s="1"/>
     </row>
     <row r="44" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C44" s="1">
         <v>1969</v>
@@ -2938,23 +2956,23 @@
         <v>154</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="G44" s="1"/>
       <c r="H44" s="1" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="I44" s="1"/>
     </row>
     <row r="45" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C45" s="1">
         <v>1970</v>
@@ -2963,23 +2981,23 @@
         <v>66</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="G45" s="1"/>
       <c r="H45" s="1" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="I45" s="1"/>
     </row>
     <row r="46" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C46" s="1">
         <v>1970</v>
@@ -2988,23 +3006,23 @@
         <v>65</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F46" s="1"/>
       <c r="G46" s="1" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="I46" s="1"/>
     </row>
     <row r="47" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C47" s="1">
         <v>1970</v>
@@ -3013,23 +3031,23 @@
         <v>99</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F47" s="1"/>
       <c r="G47" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="I47" s="1"/>
     </row>
     <row r="48" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C48" s="1">
         <v>1970</v>
@@ -3038,23 +3056,23 @@
         <v>108</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F48" s="1"/>
       <c r="G48" s="1" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="I48" s="1"/>
     </row>
     <row r="49" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="C49" s="1">
         <v>1971</v>
@@ -3063,23 +3081,23 @@
         <v>105</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="F49" s="1"/>
       <c r="G49" s="1" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="I49" s="1"/>
     </row>
     <row r="50" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C50" s="1">
         <v>1971</v>
@@ -3088,23 +3106,23 @@
         <v>89</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F50" s="1"/>
       <c r="G50" s="1" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="I50" s="1"/>
     </row>
     <row r="51" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C51" s="1">
         <v>1971</v>
@@ -3113,23 +3131,23 @@
         <v>106</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F51" s="1"/>
       <c r="G51" s="1" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="I51" s="1"/>
     </row>
     <row r="52" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C52" s="1">
         <v>1971</v>
@@ -3138,23 +3156,23 @@
         <v>104</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F52" s="1"/>
       <c r="G52" s="1" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="I52" s="1"/>
     </row>
     <row r="53" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C53" s="1">
         <v>1972</v>
@@ -3163,25 +3181,25 @@
         <v>106</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="G53" s="1"/>
       <c r="H53" s="1" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="54" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="C54" s="1">
         <v>1972</v>
@@ -3190,23 +3208,23 @@
         <v>90</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F54" s="1"/>
       <c r="G54" s="1" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="I54" s="1"/>
     </row>
     <row r="55" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C55" s="1">
         <v>1973</v>
@@ -3215,23 +3233,23 @@
         <v>124</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="F55" s="1"/>
       <c r="G55" s="1" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="I55" s="1"/>
     </row>
     <row r="56" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C56" s="1">
         <v>1973</v>
@@ -3240,23 +3258,23 @@
         <v>91</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F56" s="1"/>
       <c r="G56" s="1" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="I56" s="1"/>
     </row>
     <row r="57" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C57" s="1">
         <v>1973</v>
@@ -3265,23 +3283,23 @@
         <v>78</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="F57" s="1"/>
       <c r="G57" s="1" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="I57" s="1"/>
     </row>
     <row r="58" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C58" s="1">
         <v>1974</v>
@@ -3290,23 +3308,23 @@
         <v>315</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F58" s="1"/>
       <c r="G58" s="1" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="I58" s="1"/>
     </row>
     <row r="59" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C59" s="1">
         <v>1974</v>
@@ -3319,19 +3337,19 @@
       </c>
       <c r="F59" s="1"/>
       <c r="G59" s="1" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="I59" s="1"/>
     </row>
     <row r="60" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C60" s="1">
         <v>1975</v>
@@ -3340,23 +3358,23 @@
         <v>179</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="G60" s="1"/>
       <c r="H60" s="1" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="I60" s="1"/>
     </row>
     <row r="61" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="C61" s="1">
         <v>1975</v>
@@ -3365,23 +3383,23 @@
         <v>255</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="F61" s="1"/>
       <c r="G61" s="1" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="I61" s="1"/>
     </row>
     <row r="62" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="C62" s="1">
         <v>1976</v>
@@ -3390,23 +3408,23 @@
         <v>90</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F62" s="1"/>
       <c r="G62" s="1" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="I62" s="1"/>
     </row>
     <row r="63" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C63" s="1">
         <v>1976</v>
@@ -3415,23 +3433,23 @@
         <v>84</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="G63" s="1"/>
       <c r="H63" s="1" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I63" s="1"/>
     </row>
     <row r="64" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C64" s="1">
         <v>1976</v>
@@ -3440,23 +3458,23 @@
         <v>103</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="F64" s="1"/>
       <c r="G64" s="1" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="I64" s="1"/>
     </row>
     <row r="65" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C65" s="1">
         <v>1977</v>
@@ -3465,23 +3483,23 @@
         <v>165</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F65" s="1"/>
       <c r="G65" s="1" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="I65" s="1"/>
     </row>
     <row r="66" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C66" s="1">
         <v>1977</v>
@@ -3490,23 +3508,23 @@
         <v>106</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="F66" s="1"/>
       <c r="G66" s="1" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="I66" s="1"/>
     </row>
     <row r="67" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="C67" s="1">
         <v>1977</v>
@@ -3515,23 +3533,23 @@
         <v>100</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F67" s="1"/>
       <c r="G67" s="1" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="I67" s="1"/>
     </row>
     <row r="68" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C68" s="1">
         <v>1977</v>
@@ -3544,19 +3562,19 @@
       </c>
       <c r="F68" s="1"/>
       <c r="G68" s="1" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="H68" s="1" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="I68" s="1"/>
     </row>
     <row r="69" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C69" s="1">
         <v>1978</v>
@@ -3565,23 +3583,23 @@
         <v>131</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F69" s="1"/>
       <c r="G69" s="1" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="I69" s="1"/>
     </row>
     <row r="70" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C70" s="1">
         <v>1978</v>
@@ -3590,23 +3608,23 @@
         <v>104</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F70" s="1"/>
       <c r="G70" s="1" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="H70" s="1" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="I70" s="1"/>
     </row>
     <row r="71" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="C71" s="1">
         <v>1978</v>
@@ -3615,23 +3633,23 @@
         <v>97</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F71" s="1"/>
       <c r="G71" s="1" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="H71" s="1" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="I71" s="1"/>
     </row>
     <row r="72" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C72" s="1">
         <v>1979</v>
@@ -3640,23 +3658,23 @@
         <v>118</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="F72" s="1"/>
       <c r="G72" s="1" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="H72" s="1" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="I72" s="1"/>
     </row>
     <row r="73" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C73" s="1">
         <v>1979</v>
@@ -3665,23 +3683,23 @@
         <v>117</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F73" s="1"/>
       <c r="G73" s="1" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="H73" s="1" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="I73" s="1"/>
     </row>
     <row r="74" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C74" s="1">
         <v>1979</v>
@@ -3690,23 +3708,23 @@
         <v>115</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F74" s="1"/>
       <c r="G74" s="1" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="H74" s="1" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="I74" s="1"/>
     </row>
     <row r="75" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="C75" s="1">
         <v>1979</v>
@@ -3715,23 +3733,23 @@
         <v>92</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="F75" s="1"/>
       <c r="G75" s="1" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="H75" s="1" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="I75" s="1"/>
     </row>
     <row r="76" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="C76" s="1">
         <v>1980</v>
@@ -3740,23 +3758,23 @@
         <v>111</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="G76" s="1"/>
       <c r="H76" s="1" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="I76" s="1"/>
     </row>
     <row r="77" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C77" s="1">
         <v>1980</v>
@@ -3765,23 +3783,23 @@
         <v>90</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="F77" s="1"/>
       <c r="G77" s="1" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="H77" s="1" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="I77" s="1"/>
     </row>
     <row r="78" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C78" s="1">
         <v>1980</v>
@@ -3790,23 +3808,23 @@
         <v>116</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F78" s="1"/>
       <c r="G78" s="1" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="H78" s="1" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="I78" s="1"/>
     </row>
     <row r="79" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C79" s="1">
         <v>1981</v>
@@ -3815,23 +3833,23 @@
         <v>105</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="F79" s="1"/>
       <c r="G79" s="1" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="H79" s="1" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="I79" s="1"/>
     </row>
     <row r="80" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C80" s="1">
         <v>1981</v>
@@ -3840,23 +3858,25 @@
         <v>122</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="F80" s="1"/>
       <c r="G80" s="1" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="H80" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="I80" s="1"/>
+        <v>305</v>
+      </c>
+      <c r="I80" s="1" t="s">
+        <v>306</v>
+      </c>
     </row>
     <row r="81" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C81" s="1">
         <v>1981</v>
@@ -3865,23 +3885,23 @@
         <v>153</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F81" s="1"/>
       <c r="G81" s="1" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="H81" s="1" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="I81" s="1"/>
     </row>
     <row r="82" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="C82" s="1">
         <v>1981</v>
@@ -3890,23 +3910,23 @@
         <v>92</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="F82" s="1"/>
       <c r="G82" s="1" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="H82" s="1" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="I82" s="1"/>
     </row>
     <row r="83" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="C83" s="1">
         <v>1981</v>
@@ -3915,23 +3935,23 @@
         <v>90</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="F83" s="1"/>
       <c r="G83" s="1" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="H83" s="1" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="I83" s="1"/>
     </row>
     <row r="84" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="C84" s="1">
         <v>1982</v>
@@ -3940,23 +3960,23 @@
         <v>118</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F84" s="1"/>
       <c r="G84" s="1" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="H84" s="1" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="I84" s="1"/>
     </row>
     <row r="85" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="C85" s="1">
         <v>1982</v>
@@ -3965,23 +3985,23 @@
         <v>122</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F85" s="1"/>
       <c r="G85" s="1" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="H85" s="1" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="I85" s="1"/>
     </row>
     <row r="86" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C86" s="1">
         <v>1982</v>
@@ -3990,23 +4010,23 @@
         <v>109</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F86" s="1"/>
       <c r="G86" s="1" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="H86" s="1" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="I86" s="1"/>
     </row>
     <row r="87" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C87" s="1">
         <v>1982</v>
@@ -4015,25 +4035,25 @@
         <v>129</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F87" s="1"/>
       <c r="G87" s="1" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="H87" s="1" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="I87" s="1" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
     </row>
     <row r="88" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C88" s="1">
         <v>1982</v>
@@ -4042,23 +4062,23 @@
         <v>92</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F88" s="1"/>
       <c r="G88" s="1" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="H88" s="1" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="I88" s="1"/>
     </row>
     <row r="89" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C89" s="1">
         <v>1984</v>
@@ -4070,20 +4090,20 @@
         <v>11</v>
       </c>
       <c r="F89" s="1" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="G89" s="1"/>
       <c r="H89" s="1" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="I89" s="1"/>
     </row>
     <row r="90" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C90" s="1">
         <v>1984</v>
@@ -4092,23 +4112,23 @@
         <v>91</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="F90" s="1"/>
       <c r="G90" s="1" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="H90" s="1" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="I90" s="1"/>
     </row>
     <row r="91" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="C91" s="1">
         <v>1984</v>
@@ -4117,23 +4137,23 @@
         <v>84</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="F91" s="1"/>
       <c r="G91" s="1" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="H91" s="1" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="I91" s="1"/>
     </row>
     <row r="92" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="C92" s="1">
         <v>1985</v>
@@ -4142,23 +4162,23 @@
         <v>156</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="F92" s="1"/>
       <c r="G92" s="1" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="H92" s="1" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="I92" s="1"/>
     </row>
     <row r="93" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C93" s="1">
         <v>1985</v>
@@ -4167,23 +4187,23 @@
         <v>107</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="F93" s="1"/>
       <c r="G93" s="1" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="H93" s="1" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="I93" s="1"/>
     </row>
     <row r="94" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C94" s="1">
         <v>1987</v>
@@ -4192,23 +4212,23 @@
         <v>105</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F94" s="1" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="G94" s="1"/>
       <c r="H94" s="1" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="I94" s="1"/>
     </row>
     <row r="95" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C95" s="1">
         <v>1988</v>
@@ -4217,23 +4237,23 @@
         <v>84</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="F95" s="1"/>
       <c r="G95" s="1" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="H95" s="1" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="I95" s="1"/>
     </row>
     <row r="96" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C96" s="1">
         <v>1988</v>
@@ -4242,23 +4262,23 @@
         <v>87</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F96" s="1"/>
       <c r="G96" s="1" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="H96" s="1" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="I96" s="1"/>
     </row>
     <row r="97" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C97" s="1">
         <v>1989</v>
@@ -4267,23 +4287,23 @@
         <v>572</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="F97" s="1"/>
       <c r="G97" s="1" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="H97" s="1" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="I97" s="1"/>
     </row>
     <row r="98" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="C98" s="1">
         <v>1988</v>
@@ -4292,23 +4312,23 @@
         <v>100</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="F98" s="1"/>
       <c r="G98" s="1" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="H98" s="1" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="I98" s="1"/>
     </row>
     <row r="99" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="C99" s="1">
         <v>1988</v>
@@ -4317,23 +4337,23 @@
         <v>96</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="F99" s="1"/>
       <c r="G99" s="1" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="H99" s="1" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="I99" s="1"/>
     </row>
     <row r="100" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="C100" s="1">
         <v>1989</v>
@@ -4342,23 +4362,23 @@
         <v>100</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F100" s="1"/>
       <c r="G100" s="1" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="H100" s="1" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="I100" s="1"/>
     </row>
     <row r="101" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C101" s="1">
         <v>1991</v>
@@ -4367,23 +4387,23 @@
         <v>92</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F101" s="1" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="G101" s="1"/>
       <c r="H101" s="1" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="I101" s="1"/>
     </row>
     <row r="102" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C102" s="1">
         <v>1991</v>
@@ -4392,23 +4412,23 @@
         <v>98</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="F102" s="1"/>
       <c r="G102" s="1" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="H102" s="1" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="I102" s="1"/>
     </row>
     <row r="103" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="C103" s="1">
         <v>1992</v>
@@ -4417,23 +4437,23 @@
         <v>104</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F103" s="1" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="G103" s="1"/>
       <c r="H103" s="1" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="I103" s="1"/>
     </row>
     <row r="104" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C104" s="1">
         <v>1993</v>
@@ -4442,23 +4462,23 @@
         <v>98</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="F104" s="1"/>
       <c r="G104" s="1" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="H104" s="1" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="I104" s="1"/>
     </row>
     <row r="105" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C105" s="1">
         <v>1994</v>
@@ -4467,23 +4487,23 @@
         <v>91</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="F105" s="1"/>
       <c r="G105" s="1" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="H105" s="1" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="I105" s="1"/>
     </row>
     <row r="106" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C106" s="1">
         <v>1994</v>
@@ -4492,23 +4512,23 @@
         <v>99</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="F106" s="1"/>
       <c r="G106" s="1" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="H106" s="1" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="I106" s="1"/>
     </row>
     <row r="107" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C107" s="1">
         <v>1997</v>
@@ -4517,23 +4537,23 @@
         <v>104</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="F107" s="1"/>
       <c r="G107" s="1" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="H107" s="1" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I107" s="1"/>
     </row>
     <row r="108" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="C108" s="1">
         <v>1997</v>
@@ -4542,23 +4562,23 @@
         <v>90</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="F108" s="1"/>
       <c r="G108" s="1" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="H108" s="1" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="I108" s="1"/>
     </row>
     <row r="109" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="C109" s="1">
         <v>1999</v>
@@ -4567,23 +4587,23 @@
         <v>100</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F109" s="1"/>
       <c r="G109" s="1" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="H109" s="1" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="I109" s="1"/>
     </row>
     <row r="110" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C110" s="1">
         <v>1999</v>
@@ -4592,25 +4612,25 @@
         <v>150</v>
       </c>
       <c r="E110" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F110" s="1" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="G110" s="1"/>
       <c r="H110" s="1" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="I110" s="1" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
     </row>
     <row r="111" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C111" s="1">
         <v>1999</v>
@@ -4619,23 +4639,23 @@
         <v>175</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F111" s="1"/>
       <c r="G111" s="1" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="H111" s="1" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="I111" s="1"/>
     </row>
     <row r="112" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="C112" s="1">
         <v>2000</v>
@@ -4644,23 +4664,23 @@
         <v>98</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="F112" s="1"/>
       <c r="G112" s="1" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="H112" s="1" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="I112" s="1"/>
     </row>
     <row r="113" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="C113" s="1">
         <v>2001</v>
@@ -4669,23 +4689,23 @@
         <v>84</v>
       </c>
       <c r="E113" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F113" s="1"/>
       <c r="G113" s="1" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="H113" s="1" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="I113" s="1"/>
     </row>
     <row r="114" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="C114" s="1">
         <v>2002</v>
@@ -4694,23 +4714,23 @@
         <v>100</v>
       </c>
       <c r="E114" s="1" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="F114" s="1"/>
       <c r="G114" s="1" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="H114" s="1" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="I114" s="1"/>
     </row>
     <row r="115" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C115" s="1">
         <v>2002</v>
@@ -4719,23 +4739,23 @@
         <v>150</v>
       </c>
       <c r="E115" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F115" s="1"/>
       <c r="G115" s="1" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="H115" s="1" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="I115" s="1"/>
     </row>
     <row r="116" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="C116" s="1">
         <v>2002</v>
@@ -4744,23 +4764,23 @@
         <v>97</v>
       </c>
       <c r="E116" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F116" s="1"/>
       <c r="G116" s="1" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="H116" s="1" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="I116" s="1"/>
     </row>
     <row r="117" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="C117" s="1">
         <v>2004</v>
@@ -4769,23 +4789,23 @@
         <v>100</v>
       </c>
       <c r="E117" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F117" s="1"/>
       <c r="G117" s="1" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="H117" s="1" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="I117" s="1"/>
     </row>
     <row r="118" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="C118" s="1">
         <v>2004</v>
@@ -4794,25 +4814,25 @@
         <v>111</v>
       </c>
       <c r="E118" s="1" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="F118" s="1"/>
       <c r="G118" s="1" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="H118" s="1" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="I118" s="1" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
     </row>
     <row r="119" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="C119" s="1">
         <v>2006</v>
@@ -4821,23 +4841,23 @@
         <v>105</v>
       </c>
       <c r="E119" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F119" s="1"/>
       <c r="G119" s="1" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="H119" s="1" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="I119" s="1"/>
     </row>
     <row r="120" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C120" s="1">
         <v>2007</v>
@@ -4846,23 +4866,23 @@
         <v>118</v>
       </c>
       <c r="E120" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F120" s="1"/>
       <c r="G120" s="1" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
       <c r="H120" s="1" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="I120" s="1"/>
     </row>
     <row r="121" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="C121" s="1">
         <v>2009</v>
@@ -4871,23 +4891,23 @@
         <v>99</v>
       </c>
       <c r="E121" s="1" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F121" s="1"/>
       <c r="G121" s="1" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="H121" s="1" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="I121" s="1"/>
     </row>
     <row r="122" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="C122" s="1">
         <v>2009</v>
@@ -4896,23 +4916,23 @@
         <v>105</v>
       </c>
       <c r="E122" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F122" s="1"/>
       <c r="G122" s="1" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="H122" s="1" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
       <c r="I122" s="1"/>
     </row>
     <row r="123" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C123" s="1">
         <v>2011</v>
@@ -4921,23 +4941,23 @@
         <v>145</v>
       </c>
       <c r="E123" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F123" s="1"/>
       <c r="G123" s="1" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="H123" s="1" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="I123" s="1"/>
     </row>
     <row r="124" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="C124" s="1">
         <v>2011</v>
@@ -4946,23 +4966,23 @@
         <v>90</v>
       </c>
       <c r="E124" s="1" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="F124" s="1"/>
       <c r="G124" s="1" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="H124" s="1" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="I124" s="1"/>
     </row>
     <row r="125" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="C125" s="1">
         <v>2013</v>
@@ -4971,23 +4991,23 @@
         <v>82</v>
       </c>
       <c r="E125" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F125" s="1"/>
       <c r="G125" s="1" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="H125" s="1" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="I125" s="1"/>
     </row>
     <row r="126" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="C126" s="1">
         <v>2013</v>
@@ -4996,23 +5016,23 @@
         <v>107</v>
       </c>
       <c r="E126" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F126" s="1"/>
       <c r="G126" s="1" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="H126" s="1" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="I126" s="1"/>
     </row>
     <row r="127" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="C127" s="1">
         <v>2016</v>
@@ -5021,23 +5041,23 @@
         <v>124</v>
       </c>
       <c r="E127" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F127" s="1"/>
       <c r="G127" s="1" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="H127" s="1" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="I127" s="1"/>
     </row>
     <row r="128" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="C128" s="1">
         <v>2016</v>
@@ -5046,23 +5066,23 @@
         <v>150</v>
       </c>
       <c r="E128" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F128" s="1"/>
       <c r="G128" s="1" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="H128" s="1" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="I128" s="1"/>
     </row>
     <row r="129" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="C129" s="1">
         <v>2018</v>
@@ -5071,23 +5091,23 @@
         <v>88</v>
       </c>
       <c r="E129" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F129" s="1"/>
       <c r="G129" s="1" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="H129" s="1" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="I129" s="1"/>
     </row>
     <row r="130" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="C130" s="1">
         <v>2019</v>
@@ -5096,14 +5116,14 @@
         <v>116</v>
       </c>
       <c r="E130" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F130" s="1"/>
       <c r="G130" s="1" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="H130" s="1" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="I130" s="1"/>
     </row>

</xml_diff>

<commit_message>
lepsze cytaty, bez powielania tytulu
</commit_message>
<xml_diff>
--- a/filmy.xlsx
+++ b/filmy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/96626423858cd10c/Studia ^M kursy/Github/Movie app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_2843028F5F75A24349D9D357BABC0748EE37753E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{899B14A5-1DB6-4174-819F-9991B4F07F8F}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_2843028F24ED27460DD8D39EBAA90A02FD5D4A29" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C14A3727-781F-4D9C-9BED-C3E1862AB486}"/>
   <bookViews>
     <workbookView xWindow="-51600" yWindow="0" windowWidth="25800" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="486">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="492">
   <si>
     <t>Tytuł</t>
   </si>
@@ -58,54 +58,57 @@
     <t>Leon Trystan</t>
   </si>
   <si>
+    <t>Komedia, Musicale</t>
+  </si>
+  <si>
+    <t>Adolf Dymsza w przebraniu, które ma rozstrzygnąć spór o spokój w kamienicy.</t>
+  </si>
+  <si>
+    <t>Przedwojenna komedia o wojnie sąsiedzkiej prowadzonej przez sufit.</t>
+  </si>
+  <si>
+    <t>https://www.filmweb.pl/film/Pi%C4%99tro+wy%C5%BCej-1937-33181</t>
+  </si>
+  <si>
+    <t>Znachor</t>
+  </si>
+  <si>
+    <t>Michał Waszyński</t>
+  </si>
+  <si>
+    <t>Obyczajowe</t>
+  </si>
+  <si>
+    <t>Chirurg bez pamięci, który leczy wiejskimi sposobami i sam nie wie dlaczego.</t>
+  </si>
+  <si>
+    <t>Pierwowzór najsłynniejszego polskiego melodramatu, kręcony jeszcze przed wojną.</t>
+  </si>
+  <si>
+    <t>https://www.filmweb.pl/film/Znachor-1937-36236</t>
+  </si>
+  <si>
+    <t>Zapomniana melodia</t>
+  </si>
+  <si>
+    <t>Konrad Tom</t>
+  </si>
+  <si>
+    <t>Numery muzyczne kręcone z rozmachem, jakiego polskie kino potem długo nie miało.</t>
+  </si>
+  <si>
+    <t>Przedwojenny musical o nauczycielu gimnastyki, pensji dla dziewcząt i piosence nie do wyrzucenia z głowy.</t>
+  </si>
+  <si>
+    <t>https://www.filmweb.pl/film/Zapomniana+melodia-1938-33183</t>
+  </si>
+  <si>
+    <t>Włóczęgi</t>
+  </si>
+  <si>
     <t>Komedia</t>
   </si>
   <si>
-    <t>Adolf Dymsza w przebraniu, które ma rozstrzygnąć spór o spokój w kamienicy.</t>
-  </si>
-  <si>
-    <t>Przedwojenna komedia o wojnie sąsiedzkiej prowadzonej przez sufit.</t>
-  </si>
-  <si>
-    <t>https://www.filmweb.pl/film/Pi%C4%99tro+wy%C5%BCej-1937-33181</t>
-  </si>
-  <si>
-    <t>Znachor</t>
-  </si>
-  <si>
-    <t>Michał Waszyński</t>
-  </si>
-  <si>
-    <t>Obyczajowe</t>
-  </si>
-  <si>
-    <t>Chirurg bez pamięci, który leczy wiejskimi sposobami i sam nie wie dlaczego.</t>
-  </si>
-  <si>
-    <t>Pierwowzór najsłynniejszego polskiego melodramatu, kręcony jeszcze przed wojną.</t>
-  </si>
-  <si>
-    <t>https://www.filmweb.pl/film/Znachor-1937-36236</t>
-  </si>
-  <si>
-    <t>Zapomniana melodia</t>
-  </si>
-  <si>
-    <t>Konrad Tom</t>
-  </si>
-  <si>
-    <t>Numery muzyczne kręcone z rozmachem, jakiego polskie kino potem długo nie miało.</t>
-  </si>
-  <si>
-    <t>Przedwojenny musical o nauczycielu gimnastyki, pensji dla dziewcząt i piosence nie do wyrzucenia z głowy.</t>
-  </si>
-  <si>
-    <t>https://www.filmweb.pl/film/Zapomniana+melodia-1938-33183</t>
-  </si>
-  <si>
-    <t>Włóczęgi</t>
-  </si>
-  <si>
     <t>Szczepko i Tońko śpiewający o mieście, w którym film powstał.</t>
   </si>
   <si>
@@ -145,426 +148,429 @@
     <t>Odbudowywane miasto w tle każdego ujęcia, kręcone naprawdę.</t>
   </si>
   <si>
-    <t>Komedia mieszkaniowa w gruzach Warszawy — o parze, która szuka własnego kąta.</t>
+    <t>Komedia mieszkaniowa w gruzach Warszawy, o parze, która szuka własnego kąta.</t>
   </si>
   <si>
     <t>Przygoda na Mariensztacie</t>
   </si>
   <si>
+    <t>Komedia, PRL, Musicale</t>
+  </si>
+  <si>
+    <t>Socrealizm w technikolorze, dziś oglądany jak eksponat.</t>
+  </si>
+  <si>
+    <t>Pierwszy polski film kolorowy: musical o murarce i odbudowie stolicy.</t>
+  </si>
+  <si>
+    <t>Pokolenie</t>
+  </si>
+  <si>
+    <t>Andrzej Wajda</t>
+  </si>
+  <si>
+    <t>Podwórko, na którym polityczne wybory zaczynają się od zwykłego zauroczenia.</t>
+  </si>
+  <si>
+    <t>Debiut Wajdy: chłopak z przedmieścia wchodzi do konspiracji, bo zakochał się w łączniczce.</t>
+  </si>
+  <si>
+    <t>Cień</t>
+  </si>
+  <si>
+    <t>Jerzy Kawalerowicz</t>
+  </si>
+  <si>
+    <t>Kryminał</t>
+  </si>
+  <si>
+    <t>Ciało znalezione przy torach, od którego rozwijają się trzy różne czasy.</t>
+  </si>
+  <si>
+    <t>Trzy śledztwa w trzech epokach, spięte jednym nierozpoznanym trupem.</t>
+  </si>
+  <si>
+    <t>Kanał</t>
+  </si>
+  <si>
+    <t>Krata na wylocie kanału, za którą widać rzekę i wolność.</t>
+  </si>
+  <si>
+    <t>Powstańcy schodzą do kanałów i film zamienia się w powolne zejście bez wyjścia.</t>
+  </si>
+  <si>
+    <t>https://www.filmweb.pl/film/Kana%C5%82-1956-1117</t>
+  </si>
+  <si>
+    <t>Pętla</t>
+  </si>
+  <si>
+    <t>Wojciech Jerzy Has</t>
+  </si>
+  <si>
+    <t>Egzystencjalne</t>
+  </si>
+  <si>
+    <t>Zegar w kawiarni, który tyka głośniej niż wszystkie dialogi razem.</t>
+  </si>
+  <si>
+    <t>Jeden dzień alkoholika rozpisany na zegary, telefony i coraz węższe ulice.</t>
+  </si>
+  <si>
+    <t>Człowiek na torze</t>
+  </si>
+  <si>
+    <t>Andrzej Munk</t>
+  </si>
+  <si>
+    <t>PRL</t>
+  </si>
+  <si>
+    <t>Ta sama noc na torach, odtwarzana trzy razy z trzech niechętnych sobie perspektyw.</t>
+  </si>
+  <si>
+    <t>Śledztwo w sprawie śmierci maszynisty, w którym każdy świadek opowiada inny film.</t>
+  </si>
+  <si>
+    <t>Ewa chce spać</t>
+  </si>
+  <si>
+    <t>Tadeusz Chmielewski</t>
+  </si>
+  <si>
+    <t>Nocne miasto z bajki, gdzie komisariat działa jak biuro podróży.</t>
+  </si>
+  <si>
+    <t>Dziewczyna szuka noclegu w mieście, w którym złodzieje i policja świetnie się dogadują.</t>
+  </si>
+  <si>
+    <t>Popiół i diament</t>
+  </si>
+  <si>
+    <t>Kieliszki spirytusu zapalane po kolei za każdego poległego.</t>
+  </si>
+  <si>
+    <t>Ostatni dzień wojny, pierwszy dzień nowej władzy i chłopak, który nie wie, po co strzela.</t>
+  </si>
+  <si>
+    <t>Eroica</t>
+  </si>
+  <si>
+    <t>Wojna, Komedia</t>
+  </si>
+  <si>
+    <t>Oficer ukryty w obozie, z którego wszyscy zrobili legendę.</t>
+  </si>
+  <si>
+    <t>Dwie opowieści o bohaterstwie opowiedziane tak, że bohaterstwo się z nich osypuje.</t>
+  </si>
+  <si>
+    <t>Ostatni dzień lata</t>
+  </si>
+  <si>
+    <t>Tadeusz Konwicki</t>
+  </si>
+  <si>
+    <t>Odrzutowce przelatujące nad wydmami i przerywające każde zdanie.</t>
+  </si>
+  <si>
+    <t>Pusta plaża, dwoje ludzi, godzina rozmowy i wojna, o której nikt nie mówi wprost.</t>
+  </si>
+  <si>
+    <t>Pożegnania</t>
+  </si>
+  <si>
+    <t>Dansing sprzed września i to samo miejsce kilka lat później.</t>
+  </si>
+  <si>
+    <t>Przedwojenny romans, który po wojnie próbuje się skleić z zupełnie innych ludzi.</t>
+  </si>
+  <si>
+    <t>Pociąg</t>
+  </si>
+  <si>
+    <t>Kryminał, Obyczajowe</t>
+  </si>
+  <si>
+    <t>Tłum pasażerów polujący po polu na domniemanego mordercę.</t>
+  </si>
+  <si>
+    <t>Nocny pociąg nad morze, w którym każdy przedział ma sekret, a jeden pasażer jest ścigany.</t>
+  </si>
+  <si>
+    <t>Lotna</t>
+  </si>
+  <si>
+    <t>Szarża kawalerii na tle końca całej epoki.</t>
+  </si>
+  <si>
+    <t>Wrzesień 1939 i biała klacz, która przechodzi z rąk do rąk jak przepowiednia.</t>
+  </si>
+  <si>
+    <t>Krzyżacy</t>
+  </si>
+  <si>
+    <t>Aleksander Ford</t>
+  </si>
+  <si>
+    <t>Kostium</t>
+  </si>
+  <si>
+    <t>Dwa nagie miecze wręczone królowi przed bitwą.</t>
+  </si>
+  <si>
+    <t>Wielkie, ciężkie kino kostiumowe z Grunwaldem na finał.</t>
+  </si>
+  <si>
+    <t>Zezowate szczęście</t>
+  </si>
+  <si>
+    <t>Bohater zmieniający mundury szybciej, niż zmienia się władza.</t>
+  </si>
+  <si>
+    <t>Człowiek, który przez pół wieku próbuje trafić na właściwą stronę historii i zawsze się spóźnia.</t>
+  </si>
+  <si>
+    <t>Niewinni czarodzieje</t>
+  </si>
+  <si>
+    <t>Gra w zapałki zamiast rozmowy o uczuciach.</t>
+  </si>
+  <si>
+    <t>Jazz, motocykl i noc dwojga ludzi, którzy udają, że nic nie czują.</t>
+  </si>
+  <si>
+    <t>Do widzenia, do jutra</t>
+  </si>
+  <si>
+    <t>Janusz Morgenstern</t>
+  </si>
+  <si>
+    <t>Ruiny i nadmorskie ulice jako scenografia jednego lata.</t>
+  </si>
+  <si>
+    <t>Gdańsk, teatr studencki i wakacyjne zauroczenie, które nie ma szans.</t>
+  </si>
+  <si>
+    <t>Matka Joanna od Aniołów</t>
+  </si>
+  <si>
+    <t>Zakonnice w bieli padające na podłogę na tle czarnych ścian.</t>
+  </si>
+  <si>
+    <t>Egzorcysta i przeorysza w bielutkim klasztorze, gdzie wiara i pożądanie zamieniają się miejscami.</t>
+  </si>
+  <si>
+    <t>Nóż w wodzie</t>
+  </si>
+  <si>
+    <t>Roman Polański</t>
+  </si>
+  <si>
+    <t>Nóż wbijany w pokład między rozstawionymi palcami.</t>
+  </si>
+  <si>
+    <t>Małżeństwo, autostopowicz i jacht: trzy osoby, jedna łódka, rosnące ciśnienie.</t>
+  </si>
+  <si>
+    <t>Jak być kochaną</t>
+  </si>
+  <si>
+    <t>Wojna, Obyczajowe</t>
+  </si>
+  <si>
+    <t>Twarz kobiety w kadrze i całe życie opowiedziane w środku lotu.</t>
+  </si>
+  <si>
+    <t>Aktorka w samolocie wraca myślami do lat, w których ukrywała ukochanego.</t>
+  </si>
+  <si>
+    <t>Pasażerka</t>
+  </si>
+  <si>
+    <t>Stopklatki i komentarz wypełniające sceny, których nie zdążono nakręcić.</t>
+  </si>
+  <si>
+    <t>Nadzorczyni z obozu rozpoznaje na statku swoją dawną więźniarkę. Film niedokończony po śmierci reżysera.</t>
+  </si>
+  <si>
+    <t>Prawo i pięść</t>
+  </si>
+  <si>
+    <t>Jerzy Hoffman, Edward Skórzewski</t>
+  </si>
+  <si>
+    <t>Kryminał, Kostium</t>
+  </si>
+  <si>
+    <t>Pojedynek na pustej ulicy i piosenka, którą wszyscy znają bez filmu.</t>
+  </si>
+  <si>
+    <t>Polski western: były więzień pilnuje poniemieckiego miasteczka przed szabrownikami.</t>
+  </si>
+  <si>
+    <t>Rysopis</t>
+  </si>
+  <si>
+    <t>Jerzy Skolimowski</t>
+  </si>
+  <si>
+    <t>Pies prowadzony na sznurku przez ostatni wolny poranek.</t>
+  </si>
+  <si>
+    <t>Kilka godzin przed wojskiem, w których dwudziestoparolatek próbuje pozamykać całe swoje życie.</t>
+  </si>
+  <si>
+    <t>Rękopis znaleziony w Saragossie</t>
+  </si>
+  <si>
+    <t>Kostium, Kino osobne</t>
+  </si>
+  <si>
+    <t>Kielichy, które nad ranem okazują się czaszkami pod szubienicą.</t>
+  </si>
+  <si>
+    <t>Historia w historii w historii: hiszpańskie góry, duchy i najbardziej zakręcona konstrukcja polskiego kina.</t>
+  </si>
+  <si>
+    <t>Salto</t>
+  </si>
+  <si>
+    <t>Kino osobne</t>
+  </si>
+  <si>
+    <t>Cała wieś w transie, tańcząca jeden wspólny układ.</t>
+  </si>
+  <si>
+    <t>Obcy przyjeżdża do miasteczka i wszyscy zaczynają tańczyć. Dosłownie.</t>
+  </si>
+  <si>
+    <t>Walkower</t>
+  </si>
+  <si>
+    <t>Ring w hali fabrycznej i pociąg, który zaraz odjedzie.</t>
+  </si>
+  <si>
+    <t>Bokser amator jeździ po Polsce od walki do walki i od decyzji do decyzji.</t>
+  </si>
+  <si>
+    <t>Popioły</t>
+  </si>
+  <si>
+    <t>Kostium, Wojna</t>
+  </si>
+  <si>
+    <t>Szarża w wąwozie Samosierry pokazana jako rzeź, nie chwała.</t>
+  </si>
+  <si>
+    <t>Napoleońska epopeja bez cienia sentymentu wobec polskiego mitu żołnierskiego.</t>
+  </si>
+  <si>
+    <t>Faraon</t>
+  </si>
+  <si>
+    <t>Zaćmienie słońca użyte przez kapłanów jako broń polityczna.</t>
+  </si>
+  <si>
+    <t>Młody faraon kontra kapłani: kino o mechanice władzy, kręcone w piachu i złocie.</t>
+  </si>
+  <si>
+    <t>Bariera</t>
+  </si>
+  <si>
+    <t>Bohater zjeżdżający po zaśnieżonym mieście na walizce.</t>
+  </si>
+  <si>
+    <t>Student rzuca wszystko i idzie przez zimową Warszawę, która przestaje trzymać się realizmu.</t>
+  </si>
+  <si>
+    <t>Sami swoi</t>
+  </si>
+  <si>
+    <t>Sylwester Chęciński</t>
+  </si>
+  <si>
+    <t>Kargul, podejdź no do płota, jako i ja podchodzę.</t>
+  </si>
+  <si>
+    <t>Dwie rodziny przenoszą sąsiedzką wojnę na ziemie odzyskane i nie odpuszczają.</t>
+  </si>
+  <si>
+    <t>Westerplatte</t>
+  </si>
+  <si>
+    <t>Stanisław Różewicz</t>
+  </si>
+  <si>
+    <t>Rozmowa o tym, kiedy dalszy opór przestaje mieć sens.</t>
+  </si>
+  <si>
+    <t>Siedem dni obrony pokazanych jako praca, zmęczenie i decyzje dowódców.</t>
+  </si>
+  <si>
+    <t>Wszystko na sprzedaż</t>
+  </si>
+  <si>
+    <t>Zdjęcia, które ciągle wymykają się w stronę prawdziwej straty.</t>
+  </si>
+  <si>
+    <t>Ekipa szuka aktora, który zniknął z planu. Film o kinie i o Cybulskim.</t>
+  </si>
+  <si>
+    <t>Lalka</t>
+  </si>
+  <si>
+    <t>Sklep pełen towarów, w którym bohater przegrywa własne życie.</t>
+  </si>
+  <si>
+    <t>Wokulski, Izabela i Warszawa Prusa w wersji ciężkiej od przedmiotów i tkanin.</t>
+  </si>
+  <si>
+    <t>Struktura kryształu</t>
+  </si>
+  <si>
+    <t>Krzysztof Zanussi</t>
+  </si>
+  <si>
+    <t>Dwaj przyjaciele na zamarzniętym stawie, kłócący się o sens kariery.</t>
+  </si>
+  <si>
+    <t>Dwóch naukowców, wieś zimą i pytanie, czy wybór spokoju jest przegraną.</t>
+  </si>
+  <si>
+    <t>Sól ziemi czarnej</t>
+  </si>
+  <si>
+    <t>Kazimierz Kutz</t>
+  </si>
+  <si>
+    <t>Siedmiu braci w czerwieni i zieleni śląskiego pejzażu.</t>
+  </si>
+  <si>
+    <t>Śląskie powstanie widziane z perspektywy jednej rodziny, bardzo fizyczne, bardzo kolorowe kino.</t>
+  </si>
+  <si>
+    <t>Jak rozpętałem drugą wojnę światową</t>
+  </si>
+  <si>
+    <t>Komedia, Wojna</t>
+  </si>
+  <si>
+    <t>Grzegorz Brzęczyszczykiewicz</t>
+  </si>
+  <si>
+    <t>Franek Dolas przechodzi przez całą wojnę i wszędzie robi bałagan. Trzy części, jeden wieczór.</t>
+  </si>
+  <si>
+    <t>Rejs</t>
+  </si>
+  <si>
+    <t>Marek Piwowski</t>
+  </si>
+  <si>
     <t>Komedia, PRL</t>
   </si>
   <si>
-    <t>Socrealizm w technikolorze, dziś oglądany jak eksponat.</t>
-  </si>
-  <si>
-    <t>Pierwszy polski film kolorowy: musical o murarce i odbudowie stolicy.</t>
-  </si>
-  <si>
-    <t>Pokolenie</t>
-  </si>
-  <si>
-    <t>Andrzej Wajda</t>
-  </si>
-  <si>
-    <t>Podwórko, na którym polityczne wybory zaczynają się od zwykłego zauroczenia.</t>
-  </si>
-  <si>
-    <t>Debiut Wajdy: chłopak z przedmieścia wchodzi do konspiracji, bo zakochał się w łączniczce.</t>
-  </si>
-  <si>
-    <t>Cień</t>
-  </si>
-  <si>
-    <t>Jerzy Kawalerowicz</t>
-  </si>
-  <si>
-    <t>Kryminał</t>
-  </si>
-  <si>
-    <t>Ciało znalezione przy torach, od którego rozwijają się trzy różne czasy.</t>
-  </si>
-  <si>
-    <t>Trzy śledztwa w trzech epokach, spięte jednym nierozpoznanym trupem.</t>
-  </si>
-  <si>
-    <t>Kanał</t>
-  </si>
-  <si>
-    <t>Krata na wylocie kanału, za którą widać rzekę i wolność.</t>
-  </si>
-  <si>
-    <t>Powstańcy schodzą do kanałów i film zamienia się w powolne zejście bez wyjścia.</t>
-  </si>
-  <si>
-    <t>https://www.filmweb.pl/film/Kana%C5%82-1956-1117</t>
-  </si>
-  <si>
-    <t>Pętla</t>
-  </si>
-  <si>
-    <t>Wojciech Jerzy Has</t>
-  </si>
-  <si>
-    <t>Egzystencjalne</t>
-  </si>
-  <si>
-    <t>Zegar w kawiarni, który tyka głośniej niż wszystkie dialogi razem.</t>
-  </si>
-  <si>
-    <t>Jeden dzień alkoholika rozpisany na zegary, telefony i coraz węższe ulice.</t>
-  </si>
-  <si>
-    <t>Człowiek na torze</t>
-  </si>
-  <si>
-    <t>Andrzej Munk</t>
-  </si>
-  <si>
-    <t>PRL</t>
-  </si>
-  <si>
-    <t>Ta sama noc na torach, odtwarzana trzy razy z trzech niechętnych sobie perspektyw.</t>
-  </si>
-  <si>
-    <t>Śledztwo w sprawie śmierci maszynisty, w którym każdy świadek opowiada inny film.</t>
-  </si>
-  <si>
-    <t>Ewa chce spać</t>
-  </si>
-  <si>
-    <t>Tadeusz Chmielewski</t>
-  </si>
-  <si>
-    <t>Nocne miasto z bajki, gdzie komisariat działa jak biuro podróży.</t>
-  </si>
-  <si>
-    <t>Dziewczyna szuka noclegu w mieście, w którym złodzieje i policja świetnie się dogadują.</t>
-  </si>
-  <si>
-    <t>Popiół i diament</t>
-  </si>
-  <si>
-    <t>Kieliszki spirytusu zapalane po kolei za każdego poległego.</t>
-  </si>
-  <si>
-    <t>Ostatni dzień wojny, pierwszy dzień nowej władzy i chłopak, który nie wie, po co strzela.</t>
-  </si>
-  <si>
-    <t>Eroica</t>
-  </si>
-  <si>
-    <t>Wojna, Komedia</t>
-  </si>
-  <si>
-    <t>Oficer ukryty w obozie, z którego wszyscy zrobili legendę.</t>
-  </si>
-  <si>
-    <t>Dwie opowieści o bohaterstwie opowiedziane tak, że bohaterstwo się z nich osypuje.</t>
-  </si>
-  <si>
-    <t>Ostatni dzień lata</t>
-  </si>
-  <si>
-    <t>Tadeusz Konwicki</t>
-  </si>
-  <si>
-    <t>Odrzutowce przelatujące nad wydmami i przerywające każde zdanie.</t>
-  </si>
-  <si>
-    <t>Pusta plaża, dwoje ludzi, godzina rozmowy i wojna, o której nikt nie mówi wprost.</t>
-  </si>
-  <si>
-    <t>Pożegnania</t>
-  </si>
-  <si>
-    <t>Dansing sprzed września i to samo miejsce kilka lat później.</t>
-  </si>
-  <si>
-    <t>Przedwojenny romans, który po wojnie próbuje się skleić z zupełnie innych ludzi.</t>
-  </si>
-  <si>
-    <t>Pociąg</t>
-  </si>
-  <si>
-    <t>Kryminał, Obyczajowe</t>
-  </si>
-  <si>
-    <t>Tłum pasażerów polujący po polu na domniemanego mordercę.</t>
-  </si>
-  <si>
-    <t>Nocny pociąg nad morze, w którym każdy przedział ma sekret, a jeden pasażer jest ścigany.</t>
-  </si>
-  <si>
-    <t>Lotna</t>
-  </si>
-  <si>
-    <t>Szarża kawalerii na tle końca całej epoki.</t>
-  </si>
-  <si>
-    <t>Wrzesień 1939 i biała klacz, która przechodzi z rąk do rąk jak przepowiednia.</t>
-  </si>
-  <si>
-    <t>Krzyżacy</t>
-  </si>
-  <si>
-    <t>Aleksander Ford</t>
-  </si>
-  <si>
-    <t>Kostium</t>
-  </si>
-  <si>
-    <t>Dwa nagie miecze wręczone królowi przed bitwą.</t>
-  </si>
-  <si>
-    <t>Wielkie, ciężkie kino kostiumowe z Grunwaldem na finał.</t>
-  </si>
-  <si>
-    <t>Zezowate szczęście</t>
-  </si>
-  <si>
-    <t>Bohater zmieniający mundury szybciej, niż zmienia się władza.</t>
-  </si>
-  <si>
-    <t>Człowiek, który przez pół wieku próbuje trafić na właściwą stronę historii i zawsze się spóźnia.</t>
-  </si>
-  <si>
-    <t>Niewinni czarodzieje</t>
-  </si>
-  <si>
-    <t>Gra w zapałki zamiast rozmowy o uczuciach.</t>
-  </si>
-  <si>
-    <t>Jazz, motocykl i noc dwojga ludzi, którzy udają, że nic nie czują.</t>
-  </si>
-  <si>
-    <t>Do widzenia, do jutra</t>
-  </si>
-  <si>
-    <t>Janusz Morgenstern</t>
-  </si>
-  <si>
-    <t>Ruiny i nadmorskie ulice jako scenografia jednego lata.</t>
-  </si>
-  <si>
-    <t>Gdańsk, teatr studencki i wakacyjne zauroczenie, które nie ma szans.</t>
-  </si>
-  <si>
-    <t>Matka Joanna od Aniołów</t>
-  </si>
-  <si>
-    <t>Zakonnice w bieli padające na podłogę na tle czarnych ścian.</t>
-  </si>
-  <si>
-    <t>Egzorcysta i przeorysza w bielutkim klasztorze, gdzie wiara i pożądanie zamieniają się miejscami.</t>
-  </si>
-  <si>
-    <t>Nóż w wodzie</t>
-  </si>
-  <si>
-    <t>Roman Polański</t>
-  </si>
-  <si>
-    <t>Nóż wbijany w pokład między rozstawionymi palcami.</t>
-  </si>
-  <si>
-    <t>Małżeństwo, autostopowicz i jacht — trzy osoby, jedna łódka, rosnące ciśnienie.</t>
-  </si>
-  <si>
-    <t>Jak być kochaną</t>
-  </si>
-  <si>
-    <t>Wojna, Obyczajowe</t>
-  </si>
-  <si>
-    <t>Twarz kobiety w kadrze i całe życie opowiedziane w środku lotu.</t>
-  </si>
-  <si>
-    <t>Aktorka w samolocie wraca myślami do lat, w których ukrywała ukochanego.</t>
-  </si>
-  <si>
-    <t>Pasażerka</t>
-  </si>
-  <si>
-    <t>Stopklatki i komentarz wypełniające sceny, których nie zdążono nakręcić.</t>
-  </si>
-  <si>
-    <t>Nadzorczyni z obozu rozpoznaje na statku swoją dawną więźniarkę. Film niedokończony po śmierci reżysera.</t>
-  </si>
-  <si>
-    <t>Prawo i pięść</t>
-  </si>
-  <si>
-    <t>Jerzy Hoffman, Edward Skórzewski</t>
-  </si>
-  <si>
-    <t>Kryminał, Kostium</t>
-  </si>
-  <si>
-    <t>Pojedynek na pustej ulicy i piosenka, którą wszyscy znają bez filmu.</t>
-  </si>
-  <si>
-    <t>Polski western: były więzień pilnuje poniemieckiego miasteczka przed szabrownikami.</t>
-  </si>
-  <si>
-    <t>Rysopis</t>
-  </si>
-  <si>
-    <t>Jerzy Skolimowski</t>
-  </si>
-  <si>
-    <t>Pies prowadzony na sznurku przez ostatni wolny poranek.</t>
-  </si>
-  <si>
-    <t>Kilka godzin przed wojskiem, w których dwudziestoparolatek próbuje pozamykać całe swoje życie.</t>
-  </si>
-  <si>
-    <t>Rękopis znaleziony w Saragossie</t>
-  </si>
-  <si>
-    <t>Kostium, Kino osobne</t>
-  </si>
-  <si>
-    <t>Kielichy, które nad ranem okazują się czaszkami pod szubienicą.</t>
-  </si>
-  <si>
-    <t>Historia w historii w historii — hiszpańskie góry, duchy i najbardziej zakręcona konstrukcja polskiego kina.</t>
-  </si>
-  <si>
-    <t>Salto</t>
-  </si>
-  <si>
-    <t>Kino osobne</t>
-  </si>
-  <si>
-    <t>Cała wieś w transie, tańcząca jeden wspólny układ.</t>
-  </si>
-  <si>
-    <t>Obcy przyjeżdża do miasteczka i wszyscy zaczynają tańczyć. Dosłownie.</t>
-  </si>
-  <si>
-    <t>Walkower</t>
-  </si>
-  <si>
-    <t>Ring w hali fabrycznej i pociąg, który zaraz odjedzie.</t>
-  </si>
-  <si>
-    <t>Bokser amator jeździ po Polsce od walki do walki i od decyzji do decyzji.</t>
-  </si>
-  <si>
-    <t>Popioły</t>
-  </si>
-  <si>
-    <t>Kostium, Wojna</t>
-  </si>
-  <si>
-    <t>Szarża w wąwozie Samosierry pokazana jako rzeź, nie chwała.</t>
-  </si>
-  <si>
-    <t>Napoleońska epopeja bez cienia sentymentu wobec polskiego mitu żołnierskiego.</t>
-  </si>
-  <si>
-    <t>Faraon</t>
-  </si>
-  <si>
-    <t>Zaćmienie słońca użyte przez kapłanów jako broń polityczna.</t>
-  </si>
-  <si>
-    <t>Młody faraon kontra kapłani: kino o mechanice władzy, kręcone w piachu i złocie.</t>
-  </si>
-  <si>
-    <t>Bariera</t>
-  </si>
-  <si>
-    <t>Bohater zjeżdżający po zaśnieżonym mieście na walizce.</t>
-  </si>
-  <si>
-    <t>Student rzuca wszystko i idzie przez zimową Warszawę, która przestaje trzymać się realizmu.</t>
-  </si>
-  <si>
-    <t>Sami swoi</t>
-  </si>
-  <si>
-    <t>Sylwester Chęciński</t>
-  </si>
-  <si>
-    <t>Kargul, podejdź no do płota, jako i ja podchodzę.</t>
-  </si>
-  <si>
-    <t>Dwie rodziny przenoszą sąsiedzką wojnę na ziemie odzyskane i nie odpuszczają.</t>
-  </si>
-  <si>
-    <t>Westerplatte</t>
-  </si>
-  <si>
-    <t>Stanisław Różewicz</t>
-  </si>
-  <si>
-    <t>Rozmowa o tym, kiedy dalszy opór przestaje mieć sens.</t>
-  </si>
-  <si>
-    <t>Siedem dni obrony pokazanych jako praca, zmęczenie i decyzje dowódców.</t>
-  </si>
-  <si>
-    <t>Wszystko na sprzedaż</t>
-  </si>
-  <si>
-    <t>Zdjęcia, które ciągle wymykają się w stronę prawdziwej straty.</t>
-  </si>
-  <si>
-    <t>Ekipa szuka aktora, który zniknął z planu. Film o kinie i o Cybulskim.</t>
-  </si>
-  <si>
-    <t>Lalka</t>
-  </si>
-  <si>
-    <t>Sklep pełen towarów, w którym bohater przegrywa własne życie.</t>
-  </si>
-  <si>
-    <t>Wokulski, Izabela i Warszawa Prusa w wersji ciężkiej od przedmiotów i tkanin.</t>
-  </si>
-  <si>
-    <t>Struktura kryształu</t>
-  </si>
-  <si>
-    <t>Krzysztof Zanussi</t>
-  </si>
-  <si>
-    <t>Dwaj przyjaciele na zamarzniętym stawie, kłócący się o sens kariery.</t>
-  </si>
-  <si>
-    <t>Dwóch naukowców, wieś zimą i pytanie, czy wybór spokoju jest przegraną.</t>
-  </si>
-  <si>
-    <t>Sól ziemi czarnej</t>
-  </si>
-  <si>
-    <t>Kazimierz Kutz</t>
-  </si>
-  <si>
-    <t>Siedmiu braci w czerwieni i zieleni śląskiego pejzażu.</t>
-  </si>
-  <si>
-    <t>Śląskie powstanie widziane z perspektywy jednej rodziny — bardzo fizyczne, bardzo kolorowe kino.</t>
-  </si>
-  <si>
-    <t>Jak rozpętałem drugą wojnę światową</t>
-  </si>
-  <si>
-    <t>Komedia, Wojna</t>
-  </si>
-  <si>
-    <t>Grzegorz Brzęczyszczykiewicz</t>
-  </si>
-  <si>
-    <t>Franek Dolas przechodzi przez całą wojnę i wszędzie robi bałagan. Trzy części, jeden wieczór.</t>
-  </si>
-  <si>
-    <t>Rejs</t>
-  </si>
-  <si>
-    <t>Marek Piwowski</t>
-  </si>
-  <si>
     <t>jak mi się coś nie podoba, to ja w ogóle nie zabieram głosu</t>
   </si>
   <si>
@@ -673,7 +679,7 @@
     <t>Ojciec hodujący ptaki na strychu, w którym czas płynie wstecz.</t>
   </si>
   <si>
-    <t>Schulz przeniesiony na ekran — czas się cofa, pokoje się mnożą, wszystko pięknie gnije.</t>
+    <t>Schulz przeniesiony na ekran: czas się cofa, pokoje się mnożą, wszystko pięknie gnije.</t>
   </si>
   <si>
     <t>Iluminacja</t>
@@ -712,7 +718,7 @@
     <t>Nie ma mocnych</t>
   </si>
   <si>
-    <t>Wesele, na którym stare pretensje wracają przy każdym toaście.</t>
+    <t>Żyć nie umierać, chcą pracują, nie chcą nie pracują, demokracja człowieku!</t>
   </si>
   <si>
     <t>Kargule i Pawlaki, część druga: pojednanie idzie im równie ciężko jak wojna.</t>
@@ -841,7 +847,7 @@
     <t>Co mi zrobisz, jak mnie złapiesz</t>
   </si>
   <si>
-    <t>Zebranie, na którym każdy mówi coś innego niż myśli.</t>
+    <t>Rozpoznałem pana po znaku rozpoznawczym.</t>
   </si>
   <si>
     <t>Dyrektor, kochanka i przedsiębiorstwo, w którym nic nie działa, ale wszystko się kręci.</t>
@@ -895,7 +901,7 @@
     <t>Nie mamy pana płaszcza i co pan nam zrobi?</t>
   </si>
   <si>
-    <t>Paszport, kasa i klub sportowy Tęcza — instrukcja obsługi PRL-u w formie komedii.</t>
+    <t>Paszport, kasa i klub sportowy Tęcza: instrukcja obsługi PRL-u w formie komedii.</t>
   </si>
   <si>
     <t>Constans</t>
@@ -964,7 +970,7 @@
     <t>Studio telewizyjne jako jedyne okno na świat, w dodatku zakłamane.</t>
   </si>
   <si>
-    <t>Telewizyjny gwiazdor kontra Marsjanie — najczarniejsza polska satyra na media.</t>
+    <t>Telewizyjny gwiazdor kontra Marsjanie: najczarniejsza polska satyra na media.</t>
   </si>
   <si>
     <t>Konopielka</t>
@@ -1135,7 +1141,7 @@
     <t>Narada w hotelowym pokoju, gdzie ustala się wynik przed pierwszym gwizdkiem.</t>
   </si>
   <si>
-    <t>Sędzia, działacze i ustawiane mecze — komedia o korupcji, która nie zestarzała się ani trochę.</t>
+    <t>Sędzia, działacze i ustawiane mecze: komedia o korupcji, która nie zestarzała się ani trochę.</t>
   </si>
   <si>
     <t>Kogel-mogel</t>
@@ -1261,7 +1267,7 @@
     <t>Litwo, ojczyzno moja</t>
   </si>
   <si>
-    <t>Trzynastozgłoskowiec, który naprawdę działa na ekranie — i finałowy polonez.</t>
+    <t>Trzynastozgłoskowiec, który naprawdę działa na ekranie, i finałowy polonez.</t>
   </si>
   <si>
     <t>https://www.filmweb.pl/film/Pan+Tadeusz-1999-630</t>
@@ -1279,7 +1285,7 @@
     <t>Chłopaki nie płaczą</t>
   </si>
   <si>
-    <t>Kwartet smyczkowy próbujący zagrać koncert między jedną a drugą wpadką.</t>
+    <t>Coco jumbo i do przodu, to moje hasło.</t>
   </si>
   <si>
     <t>Studenci muzyki, gangsterzy i walizka pieniędzy, która krąży po całym mieście.</t>
@@ -1306,7 +1312,7 @@
     <t>Komedia, Egzystencjalne</t>
   </si>
   <si>
-    <t>Poranna litania przy stole: kanapka, radio i lista pretensji do świata.</t>
+    <t>Ileż to razy w myślach osiągałem wszystko. Udało mi się tylko nie być komunistą.</t>
   </si>
   <si>
     <t>Miauczyński, jego rytuały i monolog, który w duchu wygłaszał każdy mieszkaniec bloku.</t>
@@ -1481,6 +1487,18 @@
   </si>
   <si>
     <t>Chłopak po poprawczaku podszywa się pod księdza i okazuje się w tym lepszy niż powinien.</t>
+  </si>
+  <si>
+    <t>Mocne uderzenie</t>
+  </si>
+  <si>
+    <t>Jerzy Passendorfer</t>
+  </si>
+  <si>
+    <t>Skaldowie i Niebiesko-Czarni grający koncert w środku historii o pomyłce sobowtórów.</t>
+  </si>
+  <si>
+    <t>Komedia pomyłek w rytmie big-beatu, z udziałem gwiazd polskiej sceny muzycznej lat 60.</t>
   </si>
 </sst>
 </file>
@@ -1843,7 +1861,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I130"/>
+  <dimension ref="A1:I131"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1979,23 +1997,23 @@
         <v>100</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="I5" s="1"/>
     </row>
     <row r="6" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C6" s="1">
         <v>1946</v>
@@ -2004,23 +2022,23 @@
         <v>97</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I6" s="1"/>
     </row>
     <row r="7" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C7" s="1">
         <v>1948</v>
@@ -2029,23 +2047,23 @@
         <v>110</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I7" s="1"/>
     </row>
     <row r="8" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C8" s="1">
         <v>1949</v>
@@ -2054,23 +2072,23 @@
         <v>96</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I8" s="1"/>
     </row>
     <row r="9" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C9" s="1">
         <v>1954</v>
@@ -2079,23 +2097,23 @@
         <v>90</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I9" s="1"/>
     </row>
     <row r="10" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C10" s="1">
         <v>1955</v>
@@ -2104,23 +2122,23 @@
         <v>85</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F10" s="1"/>
       <c r="G10" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I10" s="1"/>
     </row>
     <row r="11" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C11" s="1">
         <v>1956</v>
@@ -2129,23 +2147,23 @@
         <v>95</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I11" s="1"/>
     </row>
     <row r="12" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C12" s="1">
         <v>1957</v>
@@ -2154,25 +2172,25 @@
         <v>91</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C13" s="1">
         <v>1957</v>
@@ -2181,23 +2199,23 @@
         <v>96</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I13" s="1"/>
     </row>
     <row r="14" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C14" s="1">
         <v>1957</v>
@@ -2206,23 +2224,23 @@
         <v>82</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I14" s="1"/>
     </row>
     <row r="15" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C15" s="1">
         <v>1957</v>
@@ -2231,23 +2249,23 @@
         <v>96</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I15" s="1"/>
     </row>
     <row r="16" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C16" s="1">
         <v>1958</v>
@@ -2256,23 +2274,23 @@
         <v>103</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I16" s="1"/>
     </row>
     <row r="17" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C17" s="1">
         <v>1958</v>
@@ -2281,23 +2299,23 @@
         <v>83</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I17" s="1"/>
     </row>
     <row r="18" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C18" s="1">
         <v>1958</v>
@@ -2310,19 +2328,19 @@
       </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I18" s="1"/>
     </row>
     <row r="19" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C19" s="1">
         <v>1958</v>
@@ -2335,19 +2353,19 @@
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="I19" s="1"/>
     </row>
     <row r="20" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C20" s="1">
         <v>1959</v>
@@ -2356,23 +2374,23 @@
         <v>93</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I20" s="1"/>
     </row>
     <row r="21" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C21" s="1">
         <v>1959</v>
@@ -2381,23 +2399,23 @@
         <v>88</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I21" s="1"/>
     </row>
     <row r="22" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C22" s="1">
         <v>1960</v>
@@ -2406,23 +2424,23 @@
         <v>166</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F22" s="1"/>
       <c r="G22" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="I22" s="1"/>
     </row>
     <row r="23" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C23" s="1">
         <v>1960</v>
@@ -2431,23 +2449,23 @@
         <v>105</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I23" s="1"/>
     </row>
     <row r="24" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C24" s="1">
         <v>1960</v>
@@ -2460,19 +2478,19 @@
       </c>
       <c r="F24" s="1"/>
       <c r="G24" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I24" s="1"/>
     </row>
     <row r="25" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C25" s="1">
         <v>1960</v>
@@ -2485,19 +2503,19 @@
       </c>
       <c r="F25" s="1"/>
       <c r="G25" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I25" s="1"/>
     </row>
     <row r="26" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C26" s="1">
         <v>1961</v>
@@ -2506,23 +2524,23 @@
         <v>110</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F26" s="1"/>
       <c r="G26" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I26" s="1"/>
     </row>
     <row r="27" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C27" s="1">
         <v>1962</v>
@@ -2535,19 +2553,19 @@
       </c>
       <c r="F27" s="1"/>
       <c r="G27" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I27" s="1"/>
     </row>
     <row r="28" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C28" s="1">
         <v>1963</v>
@@ -2556,23 +2574,23 @@
         <v>97</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F28" s="1"/>
       <c r="G28" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I28" s="1"/>
     </row>
     <row r="29" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C29" s="1">
         <v>1963</v>
@@ -2581,23 +2599,23 @@
         <v>62</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F29" s="1"/>
       <c r="G29" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I29" s="1"/>
     </row>
     <row r="30" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C30" s="1">
         <v>1964</v>
@@ -2606,23 +2624,23 @@
         <v>91</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F30" s="1"/>
       <c r="G30" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I30" s="1"/>
     </row>
     <row r="31" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C31" s="1">
         <v>1964</v>
@@ -2631,23 +2649,23 @@
         <v>76</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F31" s="1"/>
       <c r="G31" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I31" s="1"/>
     </row>
     <row r="32" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C32" s="1">
         <v>1965</v>
@@ -2656,23 +2674,23 @@
         <v>182</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F32" s="1"/>
       <c r="G32" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I32" s="1"/>
     </row>
     <row r="33" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C33" s="1">
         <v>1965</v>
@@ -2681,23 +2699,23 @@
         <v>100</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F33" s="1"/>
       <c r="G33" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I33" s="1"/>
     </row>
     <row r="34" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C34" s="1">
         <v>1965</v>
@@ -2706,23 +2724,23 @@
         <v>77</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F34" s="1"/>
       <c r="G34" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I34" s="1"/>
     </row>
     <row r="35" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C35" s="1">
         <v>1965</v>
@@ -2731,23 +2749,23 @@
         <v>233</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F35" s="1"/>
       <c r="G35" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I35" s="1"/>
     </row>
     <row r="36" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C36" s="1">
         <v>1966</v>
@@ -2756,23 +2774,23 @@
         <v>175</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F36" s="1"/>
       <c r="G36" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C37" s="1">
         <v>1966</v>
@@ -2781,23 +2799,23 @@
         <v>83</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F37" s="1"/>
       <c r="G37" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I37" s="1"/>
     </row>
     <row r="38" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C38" s="1">
         <v>1967</v>
@@ -2806,23 +2824,23 @@
         <v>87</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G38" s="1"/>
       <c r="H38" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I38" s="1"/>
     </row>
     <row r="39" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C39" s="1">
         <v>1967</v>
@@ -2831,23 +2849,23 @@
         <v>87</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F39" s="1"/>
       <c r="G39" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I39" s="1"/>
     </row>
     <row r="40" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C40" s="1">
         <v>1968</v>
@@ -2856,23 +2874,23 @@
         <v>100</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F40" s="1"/>
       <c r="G40" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I40" s="1"/>
     </row>
     <row r="41" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C41" s="1">
         <v>1968</v>
@@ -2881,23 +2899,23 @@
         <v>158</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F41" s="1"/>
       <c r="G41" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I41" s="1"/>
     </row>
     <row r="42" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C42" s="1">
         <v>1969</v>
@@ -2906,23 +2924,23 @@
         <v>74</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F42" s="1"/>
       <c r="G42" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I42" s="1"/>
     </row>
     <row r="43" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C43" s="1">
         <v>1969</v>
@@ -2931,23 +2949,23 @@
         <v>100</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F43" s="1"/>
       <c r="G43" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I43" s="1"/>
     </row>
     <row r="44" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C44" s="1">
         <v>1969</v>
@@ -2956,23 +2974,23 @@
         <v>154</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G44" s="1"/>
       <c r="H44" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I44" s="1"/>
     </row>
     <row r="45" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C45" s="1">
         <v>1970</v>
@@ -2981,23 +2999,23 @@
         <v>66</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>42</v>
+        <v>181</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="G45" s="1"/>
       <c r="H45" s="1" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="I45" s="1"/>
     </row>
     <row r="46" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C46" s="1">
         <v>1970</v>
@@ -3006,23 +3024,23 @@
         <v>65</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>42</v>
+        <v>181</v>
       </c>
       <c r="F46" s="1"/>
       <c r="G46" s="1" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="I46" s="1"/>
     </row>
     <row r="47" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C47" s="1">
         <v>1970</v>
@@ -3035,19 +3053,19 @@
       </c>
       <c r="F47" s="1"/>
       <c r="G47" s="1" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="I47" s="1"/>
     </row>
     <row r="48" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C48" s="1">
         <v>1970</v>
@@ -3056,23 +3074,23 @@
         <v>108</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F48" s="1"/>
       <c r="G48" s="1" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I48" s="1"/>
     </row>
     <row r="49" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C49" s="1">
         <v>1971</v>
@@ -3081,23 +3099,23 @@
         <v>105</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F49" s="1"/>
       <c r="G49" s="1" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="I49" s="1"/>
     </row>
     <row r="50" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C50" s="1">
         <v>1971</v>
@@ -3110,19 +3128,19 @@
       </c>
       <c r="F50" s="1"/>
       <c r="G50" s="1" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="I50" s="1"/>
     </row>
     <row r="51" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C51" s="1">
         <v>1971</v>
@@ -3131,23 +3149,23 @@
         <v>106</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>42</v>
+        <v>181</v>
       </c>
       <c r="F51" s="1"/>
       <c r="G51" s="1" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="I51" s="1"/>
     </row>
     <row r="52" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C52" s="1">
         <v>1971</v>
@@ -3156,23 +3174,23 @@
         <v>104</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F52" s="1"/>
       <c r="G52" s="1" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="I52" s="1"/>
     </row>
     <row r="53" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C53" s="1">
         <v>1972</v>
@@ -3181,25 +3199,25 @@
         <v>106</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="G53" s="1"/>
       <c r="H53" s="1" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="54" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C54" s="1">
         <v>1972</v>
@@ -3208,23 +3226,23 @@
         <v>90</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>42</v>
+        <v>181</v>
       </c>
       <c r="F54" s="1"/>
       <c r="G54" s="1" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="I54" s="1"/>
     </row>
     <row r="55" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C55" s="1">
         <v>1973</v>
@@ -3233,23 +3251,23 @@
         <v>124</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F55" s="1"/>
       <c r="G55" s="1" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="I55" s="1"/>
     </row>
     <row r="56" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C56" s="1">
         <v>1973</v>
@@ -3258,23 +3276,23 @@
         <v>91</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F56" s="1"/>
       <c r="G56" s="1" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="I56" s="1"/>
     </row>
     <row r="57" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C57" s="1">
         <v>1973</v>
@@ -3283,23 +3301,23 @@
         <v>78</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="F57" s="1"/>
       <c r="G57" s="1" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="I57" s="1"/>
     </row>
     <row r="58" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C58" s="1">
         <v>1974</v>
@@ -3308,23 +3326,23 @@
         <v>315</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F58" s="1"/>
       <c r="G58" s="1" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="I58" s="1"/>
     </row>
-    <row r="59" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C59" s="1">
         <v>1974</v>
@@ -3333,23 +3351,23 @@
         <v>100</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F59" s="1"/>
-      <c r="G59" s="1" t="s">
-        <v>229</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="G59" s="1"/>
       <c r="H59" s="1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="I59" s="1"/>
     </row>
     <row r="60" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C60" s="1">
         <v>1975</v>
@@ -3358,23 +3376,23 @@
         <v>179</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="G60" s="1"/>
       <c r="H60" s="1" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="I60" s="1"/>
     </row>
     <row r="61" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C61" s="1">
         <v>1975</v>
@@ -3383,23 +3401,23 @@
         <v>255</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="F61" s="1"/>
       <c r="G61" s="1" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="I61" s="1"/>
     </row>
     <row r="62" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C62" s="1">
         <v>1976</v>
@@ -3408,23 +3426,23 @@
         <v>90</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>42</v>
+        <v>181</v>
       </c>
       <c r="F62" s="1"/>
       <c r="G62" s="1" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="I62" s="1"/>
     </row>
     <row r="63" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C63" s="1">
         <v>1976</v>
@@ -3433,23 +3451,23 @@
         <v>84</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="G63" s="1"/>
       <c r="H63" s="1" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="I63" s="1"/>
     </row>
     <row r="64" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C64" s="1">
         <v>1976</v>
@@ -3458,23 +3476,23 @@
         <v>103</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="F64" s="1"/>
       <c r="G64" s="1" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="I64" s="1"/>
     </row>
     <row r="65" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C65" s="1">
         <v>1977</v>
@@ -3483,23 +3501,23 @@
         <v>165</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F65" s="1"/>
       <c r="G65" s="1" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="I65" s="1"/>
     </row>
     <row r="66" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C66" s="1">
         <v>1977</v>
@@ -3508,23 +3526,23 @@
         <v>106</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="F66" s="1"/>
       <c r="G66" s="1" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="I66" s="1"/>
     </row>
     <row r="67" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C67" s="1">
         <v>1977</v>
@@ -3533,23 +3551,23 @@
         <v>100</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F67" s="1"/>
       <c r="G67" s="1" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="I67" s="1"/>
     </row>
     <row r="68" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C68" s="1">
         <v>1977</v>
@@ -3558,23 +3576,23 @@
         <v>107</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F68" s="1"/>
       <c r="G68" s="1" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="H68" s="1" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="I68" s="1"/>
     </row>
     <row r="69" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C69" s="1">
         <v>1978</v>
@@ -3583,23 +3601,23 @@
         <v>131</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F69" s="1"/>
       <c r="G69" s="1" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="I69" s="1"/>
     </row>
     <row r="70" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C70" s="1">
         <v>1978</v>
@@ -3608,23 +3626,23 @@
         <v>104</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F70" s="1"/>
       <c r="G70" s="1" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="H70" s="1" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="I70" s="1"/>
     </row>
     <row r="71" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C71" s="1">
         <v>1978</v>
@@ -3633,23 +3651,23 @@
         <v>97</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F71" s="1"/>
-      <c r="G71" s="1" t="s">
-        <v>272</v>
-      </c>
+        <v>181</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="G71" s="1"/>
       <c r="H71" s="1" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="I71" s="1"/>
     </row>
     <row r="72" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C72" s="1">
         <v>1979</v>
@@ -3658,23 +3676,23 @@
         <v>118</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="F72" s="1"/>
       <c r="G72" s="1" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="H72" s="1" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="I72" s="1"/>
     </row>
     <row r="73" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C73" s="1">
         <v>1979</v>
@@ -3683,23 +3701,23 @@
         <v>117</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F73" s="1"/>
       <c r="G73" s="1" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="H73" s="1" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="I73" s="1"/>
     </row>
     <row r="74" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C74" s="1">
         <v>1979</v>
@@ -3712,19 +3730,19 @@
       </c>
       <c r="F74" s="1"/>
       <c r="G74" s="1" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="H74" s="1" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="I74" s="1"/>
     </row>
     <row r="75" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C75" s="1">
         <v>1979</v>
@@ -3733,23 +3751,23 @@
         <v>92</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F75" s="1"/>
       <c r="G75" s="1" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="H75" s="1" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="I75" s="1"/>
     </row>
     <row r="76" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C76" s="1">
         <v>1980</v>
@@ -3758,23 +3776,23 @@
         <v>111</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>42</v>
+        <v>181</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="G76" s="1"/>
       <c r="H76" s="1" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="I76" s="1"/>
     </row>
     <row r="77" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C77" s="1">
         <v>1980</v>
@@ -3783,23 +3801,23 @@
         <v>90</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="F77" s="1"/>
       <c r="G77" s="1" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="H77" s="1" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="I77" s="1"/>
     </row>
     <row r="78" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C78" s="1">
         <v>1980</v>
@@ -3808,23 +3826,23 @@
         <v>116</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F78" s="1"/>
       <c r="G78" s="1" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="H78" s="1" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="I78" s="1"/>
     </row>
     <row r="79" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C79" s="1">
         <v>1981</v>
@@ -3833,23 +3851,23 @@
         <v>105</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="F79" s="1"/>
       <c r="G79" s="1" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="H79" s="1" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="I79" s="1"/>
     </row>
     <row r="80" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C80" s="1">
         <v>1981</v>
@@ -3858,25 +3876,25 @@
         <v>122</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="F80" s="1"/>
       <c r="G80" s="1" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="H80" s="1" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="I80" s="1" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="81" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C81" s="1">
         <v>1981</v>
@@ -3885,23 +3903,23 @@
         <v>153</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F81" s="1"/>
       <c r="G81" s="1" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="H81" s="1" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="I81" s="1"/>
     </row>
     <row r="82" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C82" s="1">
         <v>1981</v>
@@ -3910,23 +3928,23 @@
         <v>92</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="F82" s="1"/>
       <c r="G82" s="1" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="H82" s="1" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="I82" s="1"/>
     </row>
     <row r="83" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="C83" s="1">
         <v>1981</v>
@@ -3935,23 +3953,23 @@
         <v>90</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="F83" s="1"/>
       <c r="G83" s="1" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="H83" s="1" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="I83" s="1"/>
     </row>
     <row r="84" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C84" s="1">
         <v>1982</v>
@@ -3960,23 +3978,23 @@
         <v>118</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F84" s="1"/>
       <c r="G84" s="1" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="H84" s="1" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="I84" s="1"/>
     </row>
     <row r="85" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C85" s="1">
         <v>1982</v>
@@ -3985,23 +4003,23 @@
         <v>122</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F85" s="1"/>
       <c r="G85" s="1" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="H85" s="1" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="I85" s="1"/>
     </row>
     <row r="86" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C86" s="1">
         <v>1982</v>
@@ -4010,14 +4028,14 @@
         <v>109</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F86" s="1"/>
       <c r="G86" s="1" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="H86" s="1" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="I86" s="1"/>
     </row>
@@ -4026,7 +4044,7 @@
         <v>15</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C87" s="1">
         <v>1982</v>
@@ -4039,21 +4057,21 @@
       </c>
       <c r="F87" s="1"/>
       <c r="G87" s="1" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="H87" s="1" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="I87" s="1" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="88" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C88" s="1">
         <v>1982</v>
@@ -4062,23 +4080,23 @@
         <v>92</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F88" s="1"/>
       <c r="G88" s="1" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="H88" s="1" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="I88" s="1"/>
     </row>
     <row r="89" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C89" s="1">
         <v>1984</v>
@@ -4087,23 +4105,23 @@
         <v>121</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F89" s="1" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="G89" s="1"/>
       <c r="H89" s="1" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="I89" s="1"/>
     </row>
     <row r="90" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C90" s="1">
         <v>1984</v>
@@ -4112,23 +4130,23 @@
         <v>91</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="F90" s="1"/>
       <c r="G90" s="1" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="H90" s="1" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="I90" s="1"/>
     </row>
     <row r="91" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C91" s="1">
         <v>1984</v>
@@ -4137,23 +4155,23 @@
         <v>84</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F91" s="1"/>
       <c r="G91" s="1" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="H91" s="1" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="I91" s="1"/>
     </row>
     <row r="92" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C92" s="1">
         <v>1985</v>
@@ -4162,23 +4180,23 @@
         <v>156</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F92" s="1"/>
       <c r="G92" s="1" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="H92" s="1" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="I92" s="1"/>
     </row>
     <row r="93" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C93" s="1">
         <v>1985</v>
@@ -4187,23 +4205,23 @@
         <v>107</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="F93" s="1"/>
       <c r="G93" s="1" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="H93" s="1" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="I93" s="1"/>
     </row>
     <row r="94" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C94" s="1">
         <v>1987</v>
@@ -4212,23 +4230,23 @@
         <v>105</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>42</v>
+        <v>181</v>
       </c>
       <c r="F94" s="1" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="G94" s="1"/>
       <c r="H94" s="1" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="I94" s="1"/>
     </row>
     <row r="95" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C95" s="1">
         <v>1988</v>
@@ -4237,23 +4255,23 @@
         <v>84</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="F95" s="1"/>
       <c r="G95" s="1" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="H95" s="1" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="I95" s="1"/>
     </row>
     <row r="96" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C96" s="1">
         <v>1988</v>
@@ -4266,19 +4284,19 @@
       </c>
       <c r="F96" s="1"/>
       <c r="G96" s="1" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="H96" s="1" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="I96" s="1"/>
     </row>
     <row r="97" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C97" s="1">
         <v>1989</v>
@@ -4287,23 +4305,23 @@
         <v>572</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="F97" s="1"/>
       <c r="G97" s="1" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="H97" s="1" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="I97" s="1"/>
     </row>
     <row r="98" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C98" s="1">
         <v>1988</v>
@@ -4312,23 +4330,23 @@
         <v>100</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="F98" s="1"/>
       <c r="G98" s="1" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="H98" s="1" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="I98" s="1"/>
     </row>
     <row r="99" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="C99" s="1">
         <v>1988</v>
@@ -4337,23 +4355,23 @@
         <v>96</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="F99" s="1"/>
       <c r="G99" s="1" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="H99" s="1" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="I99" s="1"/>
     </row>
     <row r="100" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="C100" s="1">
         <v>1989</v>
@@ -4366,19 +4384,19 @@
       </c>
       <c r="F100" s="1"/>
       <c r="G100" s="1" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H100" s="1" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="I100" s="1"/>
     </row>
     <row r="101" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C101" s="1">
         <v>1991</v>
@@ -4387,23 +4405,23 @@
         <v>92</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>42</v>
+        <v>181</v>
       </c>
       <c r="F101" s="1" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="G101" s="1"/>
       <c r="H101" s="1" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="I101" s="1"/>
     </row>
     <row r="102" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C102" s="1">
         <v>1991</v>
@@ -4412,23 +4430,23 @@
         <v>98</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="F102" s="1"/>
       <c r="G102" s="1" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="H102" s="1" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="I102" s="1"/>
     </row>
     <row r="103" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="C103" s="1">
         <v>1992</v>
@@ -4437,23 +4455,23 @@
         <v>104</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F103" s="1" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="G103" s="1"/>
       <c r="H103" s="1" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="I103" s="1"/>
     </row>
     <row r="104" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C104" s="1">
         <v>1993</v>
@@ -4462,23 +4480,23 @@
         <v>98</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="F104" s="1"/>
       <c r="G104" s="1" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="H104" s="1" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="I104" s="1"/>
     </row>
     <row r="105" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C105" s="1">
         <v>1994</v>
@@ -4487,23 +4505,23 @@
         <v>91</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="F105" s="1"/>
       <c r="G105" s="1" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="H105" s="1" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="I105" s="1"/>
     </row>
     <row r="106" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C106" s="1">
         <v>1994</v>
@@ -4512,23 +4530,23 @@
         <v>99</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="F106" s="1"/>
       <c r="G106" s="1" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="H106" s="1" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="I106" s="1"/>
     </row>
     <row r="107" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C107" s="1">
         <v>1997</v>
@@ -4537,23 +4555,23 @@
         <v>104</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="F107" s="1"/>
       <c r="G107" s="1" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="H107" s="1" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="I107" s="1"/>
     </row>
     <row r="108" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C108" s="1">
         <v>1997</v>
@@ -4562,23 +4580,23 @@
         <v>90</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="F108" s="1"/>
       <c r="G108" s="1" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="H108" s="1" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="I108" s="1"/>
     </row>
     <row r="109" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="C109" s="1">
         <v>1999</v>
@@ -4587,23 +4605,23 @@
         <v>100</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F109" s="1"/>
       <c r="G109" s="1" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="H109" s="1" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="I109" s="1"/>
     </row>
     <row r="110" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C110" s="1">
         <v>1999</v>
@@ -4612,25 +4630,25 @@
         <v>150</v>
       </c>
       <c r="E110" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F110" s="1" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="G110" s="1"/>
       <c r="H110" s="1" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="I110" s="1" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
     </row>
     <row r="111" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C111" s="1">
         <v>1999</v>
@@ -4639,23 +4657,23 @@
         <v>175</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F111" s="1"/>
       <c r="G111" s="1" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="H111" s="1" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="I111" s="1"/>
     </row>
-    <row r="112" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C112" s="1">
         <v>2000</v>
@@ -4664,23 +4682,23 @@
         <v>98</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>368</v>
-      </c>
-      <c r="F112" s="1"/>
-      <c r="G112" s="1" t="s">
-        <v>418</v>
-      </c>
+        <v>370</v>
+      </c>
+      <c r="F112" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="G112" s="1"/>
       <c r="H112" s="1" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="I112" s="1"/>
     </row>
     <row r="113" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="C113" s="1">
         <v>2001</v>
@@ -4693,19 +4711,19 @@
       </c>
       <c r="F113" s="1"/>
       <c r="G113" s="1" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="H113" s="1" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="I113" s="1"/>
     </row>
     <row r="114" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="C114" s="1">
         <v>2002</v>
@@ -4714,23 +4732,23 @@
         <v>100</v>
       </c>
       <c r="E114" s="1" t="s">
-        <v>426</v>
-      </c>
-      <c r="F114" s="1"/>
-      <c r="G114" s="1" t="s">
-        <v>427</v>
-      </c>
+        <v>428</v>
+      </c>
+      <c r="F114" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="G114" s="1"/>
       <c r="H114" s="1" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="I114" s="1"/>
     </row>
     <row r="115" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C115" s="1">
         <v>2002</v>
@@ -4739,23 +4757,23 @@
         <v>150</v>
       </c>
       <c r="E115" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F115" s="1"/>
       <c r="G115" s="1" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="H115" s="1" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="I115" s="1"/>
     </row>
     <row r="116" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C116" s="1">
         <v>2002</v>
@@ -4768,19 +4786,19 @@
       </c>
       <c r="F116" s="1"/>
       <c r="G116" s="1" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="H116" s="1" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="I116" s="1"/>
     </row>
     <row r="117" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="C117" s="1">
         <v>2004</v>
@@ -4793,19 +4811,19 @@
       </c>
       <c r="F117" s="1"/>
       <c r="G117" s="1" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="H117" s="1" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="I117" s="1"/>
     </row>
     <row r="118" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C118" s="1">
         <v>2004</v>
@@ -4814,25 +4832,25 @@
         <v>111</v>
       </c>
       <c r="E118" s="1" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="F118" s="1"/>
       <c r="G118" s="1" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="H118" s="1" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="I118" s="1" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="119" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="C119" s="1">
         <v>2006</v>
@@ -4845,19 +4863,19 @@
       </c>
       <c r="F119" s="1"/>
       <c r="G119" s="1" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="H119" s="1" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="I119" s="1"/>
     </row>
     <row r="120" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C120" s="1">
         <v>2007</v>
@@ -4866,23 +4884,23 @@
         <v>118</v>
       </c>
       <c r="E120" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F120" s="1"/>
       <c r="G120" s="1" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="H120" s="1" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="I120" s="1"/>
     </row>
     <row r="121" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="C121" s="1">
         <v>2009</v>
@@ -4891,23 +4909,23 @@
         <v>99</v>
       </c>
       <c r="E121" s="1" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="F121" s="1"/>
       <c r="G121" s="1" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="H121" s="1" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="I121" s="1"/>
     </row>
     <row r="122" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C122" s="1">
         <v>2009</v>
@@ -4916,23 +4934,23 @@
         <v>105</v>
       </c>
       <c r="E122" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F122" s="1"/>
       <c r="G122" s="1" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="H122" s="1" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="I122" s="1"/>
     </row>
     <row r="123" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C123" s="1">
         <v>2011</v>
@@ -4941,23 +4959,23 @@
         <v>145</v>
       </c>
       <c r="E123" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F123" s="1"/>
       <c r="G123" s="1" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="H123" s="1" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="I123" s="1"/>
     </row>
     <row r="124" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C124" s="1">
         <v>2011</v>
@@ -4966,23 +4984,23 @@
         <v>90</v>
       </c>
       <c r="E124" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F124" s="1"/>
       <c r="G124" s="1" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="H124" s="1" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I124" s="1"/>
     </row>
     <row r="125" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="C125" s="1">
         <v>2013</v>
@@ -4991,23 +5009,23 @@
         <v>82</v>
       </c>
       <c r="E125" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F125" s="1"/>
       <c r="G125" s="1" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="H125" s="1" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="I125" s="1"/>
     </row>
     <row r="126" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="C126" s="1">
         <v>2013</v>
@@ -5020,19 +5038,19 @@
       </c>
       <c r="F126" s="1"/>
       <c r="G126" s="1" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="H126" s="1" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="I126" s="1"/>
     </row>
     <row r="127" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C127" s="1">
         <v>2016</v>
@@ -5045,19 +5063,19 @@
       </c>
       <c r="F127" s="1"/>
       <c r="G127" s="1" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="H127" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="I127" s="1"/>
     </row>
     <row r="128" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C128" s="1">
         <v>2016</v>
@@ -5066,23 +5084,23 @@
         <v>150</v>
       </c>
       <c r="E128" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F128" s="1"/>
       <c r="G128" s="1" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="H128" s="1" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="I128" s="1"/>
     </row>
     <row r="129" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="C129" s="1">
         <v>2018</v>
@@ -5095,19 +5113,19 @@
       </c>
       <c r="F129" s="1"/>
       <c r="G129" s="1" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="H129" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="I129" s="1"/>
     </row>
     <row r="130" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="C130" s="1">
         <v>2019</v>
@@ -5116,16 +5134,39 @@
         <v>116</v>
       </c>
       <c r="E130" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F130" s="1"/>
       <c r="G130" s="1" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="H130" s="1" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="I130" s="1"/>
+    </row>
+    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>488</v>
+      </c>
+      <c r="B131" t="s">
+        <v>489</v>
+      </c>
+      <c r="C131">
+        <v>1966</v>
+      </c>
+      <c r="D131">
+        <v>78</v>
+      </c>
+      <c r="E131" t="s">
+        <v>11</v>
+      </c>
+      <c r="G131" t="s">
+        <v>490</v>
+      </c>
+      <c r="H131" t="s">
+        <v>491</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I130" xr:uid="{00000000-0009-0000-0000-000000000000}"/>

</xml_diff>

<commit_message>
aktualny arkusz, Komedia, gitignore
</commit_message>
<xml_diff>
--- a/filmy.xlsx
+++ b/filmy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/96626423858cd10c/Studia ^M kursy/Github/Movie app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_2843028F24ED27460DD8D39EBAA90A02FD5D4A29" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C14A3727-781F-4D9C-9BED-C3E1862AB486}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_2843028FE575E754FDD8D3F36AA810A4FD5D4AB2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ADE20548-8D94-4780-9839-22738280B317}"/>
   <bookViews>
     <workbookView xWindow="-51600" yWindow="0" windowWidth="25800" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -316,7 +316,7 @@
     <t>Kostium</t>
   </si>
   <si>
-    <t>Dwa nagie miecze wręczone królowi przed bitwą.</t>
+    <t>Mieczów ci u nas dostatek, ale i te przyjmuję jako wróżbę zwycięstwa.</t>
   </si>
   <si>
     <t>Wielkie, ciężkie kino kostiumowe z Grunwaldem na finał.</t>
@@ -325,7 +325,7 @@
     <t>Zezowate szczęście</t>
   </si>
   <si>
-    <t>Bohater zmieniający mundury szybciej, niż zmienia się władza.</t>
+    <t>Po pijanemu z człowieka zawsze wychodzi prawda.</t>
   </si>
   <si>
     <t>Człowiek, który przez pół wieku próbuje trafić na właściwą stronę historii i zawsze się spóźnia.</t>
@@ -556,7 +556,7 @@
     <t>Komedia, Wojna</t>
   </si>
   <si>
-    <t>Grzegorz Brzęczyszczykiewicz</t>
+    <t>Niemiecki oficer każe mu przeliterować nazwisko: Grzegorz Brzęczyszczykiewicz, głoska po głosce.</t>
   </si>
   <si>
     <t>Franek Dolas przechodzi przez całą wojnę i wszędzie robi bałagan. Trzy części, jeden wieczór.</t>
@@ -583,7 +583,7 @@
     <t>Andrzej Kondratiuk</t>
   </si>
   <si>
-    <t>Bohater prasujący koszulę przed wyruszeniem na ratunek miastu.</t>
+    <t>Komary rypią, wejdźmy do środka.</t>
   </si>
   <si>
     <t>Superbohater As broni Warszawy przed złodziejem wody. Absurd czystej próby.</t>
@@ -634,7 +634,7 @@
     <t>Nie lubię poniedziałku</t>
   </si>
   <si>
-    <t>Miasto, w którym wszystko idzie nie tak, ale w rytmie komedii.</t>
+    <t>Prawdziwy fachowiec nie zaczyna pracy w poniedziałek.</t>
   </si>
   <si>
     <t>Jeden poniedziałek w Warszawie i kilkanaście historii, które się o siebie zahaczają.</t>
@@ -751,7 +751,7 @@
     <t>Brunet wieczorową porą</t>
   </si>
   <si>
-    <t>Trup, którego nie ma, i mieszkanie pełne ludzi, którzy wiedzą lepiej.</t>
+    <t>Nie wiem, nie znam się, nie orientuję się, zarobiony jestem!</t>
   </si>
   <si>
     <t>Pomyłkowe morderstwo, sąsiedzi i cała PRL-owska logika załatwiania spraw.</t>
@@ -775,7 +775,7 @@
     <t>Obyczajowe, Kostium</t>
   </si>
   <si>
-    <t>Bal, na którym cała arystokracja patrzy w jedną stronę.</t>
+    <t>W naszej sferze zawsze będziesz trędowata.</t>
   </si>
   <si>
     <t>Melodramat wszech czasów: guwernantka, ordynat i rodzina, która nie pozwoli.</t>
@@ -817,7 +817,7 @@
     <t>Kochaj albo rzuć</t>
   </si>
   <si>
-    <t>Dwaj wąsaci gospodarze na amerykańskiej autostradzie.</t>
+    <t>Nareszcie człowiek czuje się jak sołtys: wysoko, najedzony i za nic nie odpowiada.</t>
   </si>
   <si>
     <t>Kargul i Pawlak lecą do Ameryki i wywożą tam swoją sąsiedzką wojnę.</t>
@@ -934,7 +934,7 @@
     <t>Kryminał, Komedia</t>
   </si>
   <si>
-    <t>Kwinto z trąbką i plan skoku rozpisany co do sekundy.</t>
+    <t>Uśmiechniesz się tylko raz, gdy otworzysz kasę.</t>
   </si>
   <si>
     <t>Kasiarz wychodzi z więzienia i planuje zemstę tak elegancką, że aż chce się kibicować.</t>
@@ -982,7 +982,7 @@
     <t>Komedia, Obyczajowe</t>
   </si>
   <si>
-    <t>Chłop, który boi się kosiarki bardziej niż diabła.</t>
+    <t>A Ziemia to okrągła jest, jak głowa!</t>
   </si>
   <si>
     <t>Do zabitej deskami wsi przyjeżdża nauczycielka i wszystko zaczyna się sypać.</t>
@@ -1021,7 +1021,7 @@
     <t>Jedna noc w karczmie u progu pierwszej wojny, gdy świat sztetla zbiera się ostatni raz.</t>
   </si>
   <si>
-    <t>Operacja przy lampie naftowej, rękami, które pamiętają więcej niż głowa.</t>
+    <t>Wysoki sądzie, to jest profesor Rafał Wilczur.</t>
   </si>
   <si>
     <t>Melodramat totalny: profesor traci pamięć, odzyskuje ją i wszyscy płaczą.</t>
@@ -1033,7 +1033,7 @@
     <t>Wielki Szu</t>
   </si>
   <si>
-    <t>Talia rozdawana tak, żeby widz zdążył zobaczyć oszustwo.</t>
+    <t>Graliśmy uczciwie: ty oszukiwałeś, ja oszukiwałem, wygrał lepszy.</t>
   </si>
   <si>
     <t>Karciany szuler uczy młodszego fachu i przegrywa z własną legendą.</t>
@@ -1051,7 +1051,7 @@
     <t>Vabank II, czyli riposta</t>
   </si>
   <si>
-    <t>Drugi skok, tym razem rozgrywany na oczach policji.</t>
+    <t>Kwinto, ty draniu, czekaj! To jeszcze nie koniec!</t>
   </si>
   <si>
     <t>Kramer wraca po zemstę, Kwinto odpowiada jeszcze bardziej wystudiowanym numerem.</t>
@@ -1072,7 +1072,7 @@
     <t>Janusz Majewski</t>
   </si>
   <si>
-    <t>Wielonarodowy oddział, w którym nikt nie rozumie rozkazów po niemiecku.</t>
+    <t>To jest kura, panie generale!</t>
   </si>
   <si>
     <t>Rozpadająca się armia austro-węgierska i garstka żołnierzy, którzy chcą po prostu wrócić do domu.</t>
@@ -1138,7 +1138,7 @@
     <t>Komedia, Kryminał</t>
   </si>
   <si>
-    <t>Narada w hotelowym pokoju, gdzie ustala się wynik przed pierwszym gwizdkiem.</t>
+    <t>Węgiel to polskie sumienie, a piłka to też polskie sumienie.</t>
   </si>
   <si>
     <t>Sędzia, działacze i ustawiane mecze: komedia o korupcji, która nie zestarzała się ani trochę.</t>
@@ -1150,7 +1150,7 @@
     <t>Roman Załuski</t>
   </si>
   <si>
-    <t>Wiejski dom i miejskie mieszkanie sfilmowane jak dwie różne planety.</t>
+    <t>Jak mówię, to mówię, a jak mówię, to wiem.</t>
   </si>
   <si>
     <t>Dziewczyna ze wsi idzie na studia i zderza się z miejskimi manierami.</t>
@@ -1231,7 +1231,7 @@
     <t>Kiler</t>
   </si>
   <si>
-    <t>Gangsterzy traktujący przypadkowego człowieka jak legendę półświatka.</t>
+    <t>Panowie, to jest jakaś pomyłka! Pomyłka? Moja żona miała na drugie „pomyłka"…</t>
   </si>
   <si>
     <t>Taksówkarz zostaje wzięty za płatnego mordercę i cała Polska w to wierzy.</t>
@@ -1243,7 +1243,7 @@
     <t>Olaf Lubaszenko</t>
   </si>
   <si>
-    <t>Retro-Warszawa i przekręt rozpisany jak numer estradowy.</t>
+    <t>Jak się nie wie, co się gra, to się gra jeden-dwa.</t>
   </si>
   <si>
     <t>Dwaj cwaniacy w latach 60. wymyślają przekręt większy od siebie.</t>
@@ -1276,7 +1276,7 @@
     <t>Ogniem i mieczem</t>
   </si>
   <si>
-    <t>Oblężenie Zbaraża kręcone z liczbą statystów nie do powtórzenia.</t>
+    <t>Mamy gości, mości panowie!</t>
   </si>
   <si>
     <t>Sienkiewicz z rozmachem: Skrzetuski, Bohun i wojna, w której nikt nie ma czystych rąk.</t>
@@ -1375,7 +1375,7 @@
     <t>Katyń</t>
   </si>
   <si>
-    <t>Lista nazwisk czytana z ambony i kobiety liczące dni.</t>
+    <t>Guziki. Zostaną po nas tylko guziki.</t>
   </si>
   <si>
     <t>Historia opowiedziana od strony rodzin, które przez lata czekały na wiadomość.</t>
@@ -1399,7 +1399,7 @@
     <t>Dom zły</t>
   </si>
   <si>
-    <t>Śnieg, wódka i milicyjny protokół spisywany w środku niczego.</t>
+    <t>Uciekaj, bo cię zabiją. Zabiją cię, jak będziesz uciekał.</t>
   </si>
   <si>
     <t>Zimowa wizja lokalna, w której zeznania nie chcą się złożyć w jedną noc.</t>
@@ -2410,7 +2410,7 @@
       </c>
       <c r="I21" s="1"/>
     </row>
-    <row r="22" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>94</v>
       </c>
@@ -2426,10 +2426,10 @@
       <c r="E22" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1" t="s">
+      <c r="F22" s="1" t="s">
         <v>97</v>
       </c>
+      <c r="G22" s="1"/>
       <c r="H22" s="1" t="s">
         <v>98</v>
       </c>
@@ -2451,10 +2451,10 @@
       <c r="E23" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1" t="s">
+      <c r="F23" s="1" t="s">
         <v>100</v>
       </c>
+      <c r="G23" s="1"/>
       <c r="H23" s="1" t="s">
         <v>101</v>
       </c>
@@ -2960,7 +2960,7 @@
       </c>
       <c r="I43" s="1"/>
     </row>
-    <row r="44" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" ht="57" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>175</v>
       </c>
@@ -2976,10 +2976,10 @@
       <c r="E44" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="F44" s="1" t="s">
+      <c r="F44" s="1"/>
+      <c r="G44" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="G44" s="1"/>
       <c r="H44" s="1" t="s">
         <v>178</v>
       </c>
@@ -3026,10 +3026,10 @@
       <c r="E46" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="F46" s="1"/>
-      <c r="G46" s="1" t="s">
+      <c r="F46" s="1" t="s">
         <v>186</v>
       </c>
+      <c r="G46" s="1"/>
       <c r="H46" s="1" t="s">
         <v>187</v>
       </c>
@@ -3151,10 +3151,10 @@
       <c r="E51" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="F51" s="1"/>
-      <c r="G51" s="1" t="s">
+      <c r="F51" s="1" t="s">
         <v>203</v>
       </c>
+      <c r="G51" s="1"/>
       <c r="H51" s="1" t="s">
         <v>204</v>
       </c>
@@ -3428,10 +3428,10 @@
       <c r="E62" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="F62" s="1"/>
-      <c r="G62" s="1" t="s">
+      <c r="F62" s="1" t="s">
         <v>242</v>
       </c>
+      <c r="G62" s="1"/>
       <c r="H62" s="1" t="s">
         <v>243</v>
       </c>
@@ -3478,10 +3478,10 @@
       <c r="E64" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="F64" s="1"/>
-      <c r="G64" s="1" t="s">
+      <c r="F64" s="1" t="s">
         <v>250</v>
       </c>
+      <c r="G64" s="1"/>
       <c r="H64" s="1" t="s">
         <v>251</v>
       </c>
@@ -3562,7 +3562,7 @@
       </c>
       <c r="I67" s="1"/>
     </row>
-    <row r="68" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>263</v>
       </c>
@@ -3578,10 +3578,10 @@
       <c r="E68" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F68" s="1"/>
-      <c r="G68" s="1" t="s">
+      <c r="F68" s="1" t="s">
         <v>264</v>
       </c>
+      <c r="G68" s="1"/>
       <c r="H68" s="1" t="s">
         <v>265</v>
       </c>
@@ -3853,10 +3853,10 @@
       <c r="E79" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="F79" s="1"/>
-      <c r="G79" s="1" t="s">
+      <c r="F79" s="1" t="s">
         <v>303</v>
       </c>
+      <c r="G79" s="1"/>
       <c r="H79" s="1" t="s">
         <v>304</v>
       </c>
@@ -3955,10 +3955,10 @@
       <c r="E83" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="F83" s="1"/>
-      <c r="G83" s="1" t="s">
+      <c r="F83" s="1" t="s">
         <v>319</v>
       </c>
+      <c r="G83" s="1"/>
       <c r="H83" s="1" t="s">
         <v>320</v>
       </c>
@@ -4039,7 +4039,7 @@
       </c>
       <c r="I86" s="1"/>
     </row>
-    <row r="87" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>15</v>
       </c>
@@ -4055,10 +4055,10 @@
       <c r="E87" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F87" s="1"/>
-      <c r="G87" s="1" t="s">
+      <c r="F87" s="1" t="s">
         <v>332</v>
       </c>
+      <c r="G87" s="1"/>
       <c r="H87" s="1" t="s">
         <v>333</v>
       </c>
@@ -4066,7 +4066,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="88" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:9" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>335</v>
       </c>
@@ -4082,10 +4082,10 @@
       <c r="E88" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F88" s="1"/>
-      <c r="G88" s="1" t="s">
+      <c r="F88" s="1" t="s">
         <v>336</v>
       </c>
+      <c r="G88" s="1"/>
       <c r="H88" s="1" t="s">
         <v>337</v>
       </c>
@@ -4132,10 +4132,10 @@
       <c r="E90" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="F90" s="1"/>
-      <c r="G90" s="1" t="s">
+      <c r="F90" s="1" t="s">
         <v>342</v>
       </c>
+      <c r="G90" s="1"/>
       <c r="H90" s="1" t="s">
         <v>343</v>
       </c>
@@ -4182,10 +4182,10 @@
       <c r="E92" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="F92" s="1"/>
-      <c r="G92" s="1" t="s">
+      <c r="F92" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="G92" s="1"/>
       <c r="H92" s="1" t="s">
         <v>350</v>
       </c>
@@ -4332,10 +4332,10 @@
       <c r="E98" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="F98" s="1"/>
-      <c r="G98" s="1" t="s">
+      <c r="F98" s="1" t="s">
         <v>371</v>
       </c>
+      <c r="G98" s="1"/>
       <c r="H98" s="1" t="s">
         <v>372</v>
       </c>
@@ -4357,10 +4357,10 @@
       <c r="E99" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="F99" s="1"/>
-      <c r="G99" s="1" t="s">
+      <c r="F99" s="1" t="s">
         <v>375</v>
       </c>
+      <c r="G99" s="1"/>
       <c r="H99" s="1" t="s">
         <v>376</v>
       </c>
@@ -4557,10 +4557,10 @@
       <c r="E107" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="F107" s="1"/>
-      <c r="G107" s="1" t="s">
+      <c r="F107" s="1" t="s">
         <v>402</v>
       </c>
+      <c r="G107" s="1"/>
       <c r="H107" s="1" t="s">
         <v>403</v>
       </c>
@@ -4582,10 +4582,10 @@
       <c r="E108" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="F108" s="1"/>
-      <c r="G108" s="1" t="s">
+      <c r="F108" s="1" t="s">
         <v>406</v>
       </c>
+      <c r="G108" s="1"/>
       <c r="H108" s="1" t="s">
         <v>407</v>
       </c>
@@ -4659,10 +4659,10 @@
       <c r="E111" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="F111" s="1"/>
-      <c r="G111" s="1" t="s">
+      <c r="F111" s="1" t="s">
         <v>417</v>
       </c>
+      <c r="G111" s="1"/>
       <c r="H111" s="1" t="s">
         <v>418</v>
       </c>
@@ -4886,10 +4886,10 @@
       <c r="E120" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="F120" s="1"/>
-      <c r="G120" s="1" t="s">
+      <c r="F120" s="1" t="s">
         <v>450</v>
       </c>
+      <c r="G120" s="1"/>
       <c r="H120" s="1" t="s">
         <v>451</v>
       </c>
@@ -4936,10 +4936,10 @@
       <c r="E122" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F122" s="1"/>
-      <c r="G122" s="1" t="s">
+      <c r="F122" s="1" t="s">
         <v>458</v>
       </c>
+      <c r="G122" s="1"/>
       <c r="H122" s="1" t="s">
         <v>459</v>
       </c>

</xml_diff>

<commit_message>
usuniete pozostale dlugie myslniki w cytatach
</commit_message>
<xml_diff>
--- a/filmy.xlsx
+++ b/filmy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/96626423858cd10c/Studia ^M kursy/Github/Movie app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_2843028FE575E754FDD8D3F36AA810A4FD5D4AB2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ADE20548-8D94-4780-9839-22738280B317}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_2843028F860DE27A55D9D3002AEA2576FC5D4B42" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7BF34C08-054E-4FAA-B41E-93D7B05CC850}"/>
   <bookViews>
     <workbookView xWindow="-51600" yWindow="0" windowWidth="25800" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -763,7 +763,7 @@
     <t>Kryminał, PRL</t>
   </si>
   <si>
-    <t>Rozbieraj się! – Tak od razu? Może najpierw buzi?</t>
+    <t>Rozbieraj się! Tak od razu? Może najpierw buzi?</t>
   </si>
   <si>
     <t>Milicyjne śledztwo pokazane od kuchni, z humorem, od którego robi się nieprzyjemnie.</t>
@@ -1093,7 +1093,7 @@
     <t>Kingsajz</t>
   </si>
   <si>
-    <t>Świeże macie muchy? – Z dzisiejszej pajęczynki.</t>
+    <t>Świeże macie muchy? Z dzisiejszej pajęczynki.</t>
   </si>
   <si>
     <t>Krasnoludki chcą urosnąć, a Szuflandia jest podejrzanie podobna do państwa obok.</t>
@@ -1533,7 +1533,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.499984740745262"/>
+        <fgColor theme="1" tint="0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>

</xml_diff>